<commit_message>
Reproducibility: run_all.sh in dependency order; scripts for S6/S9/S10; S7 no longer overwritten; PFI proportional-hazards test; batch tie-break sensitivity
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S10_Table.xlsx
+++ b/figures/supporting_information/S10_Table.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth pattern and model type" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth pattern and model type" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,74 +426,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Gene</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Lineage</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>coef_unadjusted</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>coef_growth_adjusted</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>p_growth_adjusted_two_sided</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>median_diff_excl_engineered</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>p_excl_engineered_one_sided</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>n_target_excl_engineered</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>n_suspension_comparator</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>median_diff_vs_suspension</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>p_vs_suspension_one_sided</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Gene_symbol</t>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Post-selection diagnostics of the 94 prioritised pairs; q-values are Benjamini-Hochberg adjusted within the 94 pairs (q_vs_suspension: within the 39 testable lymphoid/myeloid pairs) and are conditional on the selection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Growth pattern (Model.csv GrowthPattern: adherent, suspension, mixed, unknown) added as a categorical covariate; engineered or drug-adapted models = EngineeredModel annotated in Model.csv (10 models).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Suspension comparison: lymphoid/myeloid target lineage versus non-blood cell lines annotated as suspension cultures (41 lines); at least ten comparator lines with data required.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P95"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Lineage</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>coef_unadjusted</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>coef_growth_adjusted</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>p_growth_adjusted_two_sided</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>q_growth_adjusted</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>median_target_excl_engineered</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>median_diff_excl_engineered</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>p_excl_engineered_one_sided</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>q_excl_engineered</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>n_target_excl_engineered</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>n_suspension_comparator</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>median_diff_vs_suspension</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>p_vs_suspension_one_sided</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>q_vs_suspension</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Gene_symbol</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>KRAS (3845)</t>
         </is>
       </c>
@@ -511,18 +574,28 @@
         <v>1.643433183919731e-59</v>
       </c>
       <c r="F2" t="n">
+        <v>2.574711988140911e-58</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-2.086661855015164</v>
+      </c>
+      <c r="H2" t="n">
         <v>-1.583870584342049</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>4.414593127912001e-22</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
+        <v>2.18406186328278e-21</v>
+      </c>
+      <c r="K2" t="n">
         <v>48</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>KRAS</t>
         </is>
@@ -549,18 +622,28 @@
         <v>3.442602794463395e-152</v>
       </c>
       <c r="F3" t="n">
+        <v>3.236046626795591e-150</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-1.670194030844392</v>
+      </c>
+      <c r="H3" t="n">
         <v>-1.374409439564973</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>1.045195768518303e-27</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
+        <v>8.931672930974592e-27</v>
+      </c>
+      <c r="K3" t="n">
         <v>68</v>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>SOX10</t>
         </is>
@@ -587,18 +670,28 @@
         <v>1.122464150335925e-40</v>
       </c>
       <c r="F4" t="n">
+        <v>1.17235144590641e-39</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-1.425133103283988</v>
+      </c>
+      <c r="H4" t="n">
         <v>-1.265178331743293</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>9.418195094943622e-11</v>
       </c>
-      <c r="H4" t="n">
+      <c r="J4" t="n">
+        <v>2.213275847311751e-10</v>
+      </c>
+      <c r="K4" t="n">
         <v>34</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
         <is>
           <t>HNF1B</t>
         </is>
@@ -625,18 +718,28 @@
         <v>1.056809636006767e-15</v>
       </c>
       <c r="F5" t="n">
+        <v>6.208756611539757e-15</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-1.363840520951394</v>
+      </c>
+      <c r="H5" t="n">
         <v>-1.241998082549389</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>0.0001641540610822</v>
       </c>
-      <c r="H5" t="n">
+      <c r="J5" t="n">
+        <v>0.0001881766066064244</v>
+      </c>
+      <c r="K5" t="n">
         <v>5</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
         <is>
           <t>FOXA1</t>
         </is>
@@ -663,18 +766,28 @@
         <v>1.913639539971504e-07</v>
       </c>
       <c r="F6" t="n">
+        <v>4.612361968136446e-07</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-1.55427191249818</v>
+      </c>
+      <c r="H6" t="n">
         <v>-1.135648494549984</v>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>8.777580349667754e-06</v>
       </c>
-      <c r="H6" t="n">
+      <c r="J6" t="n">
+        <v>1.162102187139111e-05</v>
+      </c>
+      <c r="K6" t="n">
         <v>10</v>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
         <is>
           <t>MDM2</t>
         </is>
@@ -701,18 +814,28 @@
         <v>4.986058889767983e-92</v>
       </c>
       <c r="F7" t="n">
+        <v>9.373790712763807e-91</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-1.255339207492288</v>
+      </c>
+      <c r="H7" t="n">
         <v>-1.12237392801801</v>
       </c>
-      <c r="G7" t="n">
+      <c r="I7" t="n">
         <v>1.555249728656573e-25</v>
       </c>
-      <c r="H7" t="n">
+      <c r="J7" t="n">
+        <v>1.124565188413214e-24</v>
+      </c>
+      <c r="K7" t="n">
         <v>63</v>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
         <is>
           <t>CTNNB1</t>
         </is>
@@ -739,18 +862,28 @@
         <v>2.994953655844778e-15</v>
       </c>
       <c r="F8" t="n">
+        <v>1.564031353607828e-14</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-1.630766279564239</v>
+      </c>
+      <c r="H8" t="n">
         <v>-1.07582002891723</v>
       </c>
-      <c r="G8" t="n">
-        <v>8.069526804470387e-10</v>
-      </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
+        <v>8.069526804470385e-10</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1.613905360894077e-09</v>
+      </c>
+      <c r="K8" t="n">
         <v>34</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
         <is>
           <t>CFLAR</t>
         </is>
@@ -777,24 +910,36 @@
         <v>2.597573811120073e-46</v>
       </c>
       <c r="F9" t="n">
+        <v>3.052149228066087e-45</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-1.360154978943165</v>
+      </c>
+      <c r="H9" t="n">
         <v>-1.066850897578272</v>
       </c>
-      <c r="G9" t="n">
+      <c r="I9" t="n">
         <v>2.04135662657397e-25</v>
       </c>
-      <c r="H9" t="n">
+      <c r="J9" t="n">
+        <v>1.370625163556809e-24</v>
+      </c>
+      <c r="K9" t="n">
         <v>42</v>
       </c>
-      <c r="I9" t="n">
+      <c r="L9" t="n">
         <v>41</v>
       </c>
-      <c r="J9" t="n">
+      <c r="M9" t="n">
         <v>-1.033011407986264</v>
       </c>
-      <c r="K9" t="n">
-        <v>3.687172576957461e-14</v>
-      </c>
-      <c r="L9" t="inlineStr">
+      <c r="N9" t="n">
+        <v>3.687172576957462e-14</v>
+      </c>
+      <c r="O9" t="n">
+        <v>7.18998652506705e-13</v>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t>MYB</t>
         </is>
@@ -821,24 +966,36 @@
         <v>5.211680712421602e-15</v>
       </c>
       <c r="F10" t="n">
+        <v>2.449489934838153e-14</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-1.23964073579391</v>
+      </c>
+      <c r="H10" t="n">
         <v>-1.093531285888063</v>
       </c>
-      <c r="G10" t="n">
+      <c r="I10" t="n">
         <v>1.003523852663911e-20</v>
       </c>
-      <c r="H10" t="n">
+      <c r="J10" t="n">
+        <v>4.491963911924173e-20</v>
+      </c>
+      <c r="K10" t="n">
         <v>42</v>
       </c>
-      <c r="I10" t="n">
+      <c r="L10" t="n">
         <v>41</v>
       </c>
-      <c r="J10" t="n">
+      <c r="M10" t="n">
         <v>-0.9960517864762388</v>
       </c>
-      <c r="K10" t="n">
-        <v>6.409917563617628e-13</v>
-      </c>
-      <c r="L10" t="inlineStr">
+      <c r="N10" t="n">
+        <v>6.40991756361763e-13</v>
+      </c>
+      <c r="O10" t="n">
+        <v>8.332892832702918e-12</v>
+      </c>
+      <c r="P10" t="inlineStr">
         <is>
           <t>CBFB</t>
         </is>
@@ -865,18 +1022,28 @@
         <v>1.397146005251066e-07</v>
       </c>
       <c r="F11" t="n">
+        <v>3.45609801298948e-07</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-1.371058348815747</v>
+      </c>
+      <c r="H11" t="n">
         <v>-1.051640460586594</v>
       </c>
-      <c r="G11" t="n">
+      <c r="I11" t="n">
         <v>0.0002808587124174</v>
       </c>
-      <c r="H11" t="n">
+      <c r="J11" t="n">
+        <v>0.0003069851042701814</v>
+      </c>
+      <c r="K11" t="n">
         <v>5</v>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
         <is>
           <t>TUBB4B</t>
         </is>
@@ -903,18 +1070,28 @@
         <v>1.306927087769899e-47</v>
       </c>
       <c r="F12" t="n">
+        <v>1.755016375005293e-46</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-1.119002902546843</v>
+      </c>
+      <c r="H12" t="n">
         <v>-1.013443179537026</v>
       </c>
-      <c r="G12" t="n">
+      <c r="I12" t="n">
         <v>4.711894769167349e-14</v>
       </c>
-      <c r="H12" t="n">
+      <c r="J12" t="n">
+        <v>1.581850386791896e-13</v>
+      </c>
+      <c r="K12" t="n">
         <v>34</v>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
         <is>
           <t>PAX8</t>
         </is>
@@ -941,18 +1118,28 @@
         <v>1.17976165263478e-103</v>
       </c>
       <c r="F13" t="n">
+        <v>5.544879767383465e-102</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-1.124780833992745</v>
+      </c>
+      <c r="H13" t="n">
         <v>-1.039340981263017</v>
       </c>
-      <c r="G13" t="n">
+      <c r="I13" t="n">
         <v>1.72192720245487e-22</v>
       </c>
-      <c r="H13" t="n">
+      <c r="J13" t="n">
+        <v>8.992286501708766e-22</v>
+      </c>
+      <c r="K13" t="n">
         <v>68</v>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr">
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
         <is>
           <t>BRAF</t>
         </is>
@@ -979,18 +1166,28 @@
         <v>2.846253139062331e-100</v>
       </c>
       <c r="F14" t="n">
+        <v>8.918259835728637e-99</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-1.101619065138771</v>
+      </c>
+      <c r="H14" t="n">
         <v>-0.9881116948117854</v>
       </c>
-      <c r="G14" t="n">
+      <c r="I14" t="n">
         <v>6.599495954428033e-10</v>
       </c>
-      <c r="H14" t="n">
+      <c r="J14" t="n">
+        <v>1.348592651557033e-09</v>
+      </c>
+      <c r="K14" t="n">
         <v>18</v>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr">
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
         <is>
           <t>ZER1</t>
         </is>
@@ -1017,24 +1214,36 @@
         <v>5.199182551965316e-30</v>
       </c>
       <c r="F15" t="n">
+        <v>4.887231598847397e-29</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-1.200224825187052</v>
+      </c>
+      <c r="H15" t="n">
         <v>-0.957084097378387</v>
       </c>
-      <c r="G15" t="n">
+      <c r="I15" t="n">
         <v>1.246057873355729e-40</v>
       </c>
-      <c r="H15" t="n">
+      <c r="J15" t="n">
+        <v>5.856472004771927e-39</v>
+      </c>
+      <c r="K15" t="n">
         <v>94</v>
       </c>
-      <c r="I15" t="n">
+      <c r="L15" t="n">
         <v>41</v>
       </c>
-      <c r="J15" t="n">
+      <c r="M15" t="n">
         <v>-0.7924728137867726</v>
       </c>
-      <c r="K15" t="n">
-        <v>5.203690462565467e-10</v>
-      </c>
-      <c r="L15" t="inlineStr">
+      <c r="N15" t="n">
+        <v>5.203690462565465e-10</v>
+      </c>
+      <c r="O15" t="n">
+        <v>2.029439280400532e-09</v>
+      </c>
+      <c r="P15" t="inlineStr">
         <is>
           <t>NMNAT1</t>
         </is>
@@ -1061,24 +1270,36 @@
         <v>1.871900046127947e-92</v>
       </c>
       <c r="F16" t="n">
+        <v>4.398965108400675e-91</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-1.041153941289623</v>
+      </c>
+      <c r="H16" t="n">
         <v>-0.9434318573510538</v>
       </c>
-      <c r="G16" t="n">
-        <v>6.752672780856972e-29</v>
-      </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
+        <v>6.752672780856971e-29</v>
+      </c>
+      <c r="J16" t="n">
+        <v>7.05279157111728e-28</v>
+      </c>
+      <c r="K16" t="n">
         <v>94</v>
       </c>
-      <c r="I16" t="n">
+      <c r="L16" t="n">
         <v>41</v>
       </c>
-      <c r="J16" t="n">
+      <c r="M16" t="n">
         <v>-0.9445913701184904</v>
       </c>
-      <c r="K16" t="n">
+      <c r="N16" t="n">
         <v>2.538115592903102e-09</v>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="O16" t="n">
+        <v>8.248875676935083e-09</v>
+      </c>
+      <c r="P16" t="inlineStr">
         <is>
           <t>IRF4</t>
         </is>
@@ -1105,18 +1326,28 @@
         <v>8.823360352502614e-06</v>
       </c>
       <c r="F17" t="n">
+        <v>1.648247543586321e-05</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-1.978953338506378</v>
+      </c>
+      <c r="H17" t="n">
         <v>-0.9311684551737158</v>
       </c>
-      <c r="G17" t="n">
+      <c r="I17" t="n">
         <v>1.088762746783158e-07</v>
       </c>
-      <c r="H17" t="n">
+      <c r="J17" t="n">
+        <v>1.795503477151173e-07</v>
+      </c>
+      <c r="K17" t="n">
         <v>47</v>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr">
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
         <is>
           <t>CCND1</t>
         </is>
@@ -1143,18 +1374,28 @@
         <v>1.475890482115414e-09</v>
       </c>
       <c r="F18" t="n">
+        <v>4.954775189958891e-09</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-1.402905363847756</v>
+      </c>
+      <c r="H18" t="n">
         <v>-0.9237690916376592</v>
       </c>
-      <c r="G18" t="n">
+      <c r="I18" t="n">
         <v>3.127835539651249e-09</v>
       </c>
-      <c r="H18" t="n">
+      <c r="J18" t="n">
+        <v>5.880330814544348e-09</v>
+      </c>
+      <c r="K18" t="n">
         <v>34</v>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr">
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -1181,18 +1422,28 @@
         <v>7.313612224191613e-14</v>
       </c>
       <c r="F19" t="n">
+        <v>3.124907041245508e-13</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-1.569685120222577</v>
+      </c>
+      <c r="H19" t="n">
         <v>-0.9092982996204988</v>
       </c>
-      <c r="G19" t="n">
+      <c r="I19" t="n">
         <v>1.590749614014025e-06</v>
       </c>
-      <c r="H19" t="n">
+      <c r="J19" t="n">
+        <v>2.198977407607622e-06</v>
+      </c>
+      <c r="K19" t="n">
         <v>18</v>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr">
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
         <is>
           <t>SKP2</t>
         </is>
@@ -1219,18 +1470,28 @@
         <v>1.343649811283425e-11</v>
       </c>
       <c r="F20" t="n">
+        <v>5.052123290425679e-11</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-1.285985398539891</v>
+      </c>
+      <c r="H20" t="n">
         <v>-0.8707089148182607</v>
       </c>
-      <c r="G20" t="n">
+      <c r="I20" t="n">
         <v>3.204937365642594e-09</v>
       </c>
-      <c r="H20" t="n">
+      <c r="J20" t="n">
+        <v>5.907139458243213e-09</v>
+      </c>
+      <c r="K20" t="n">
         <v>34</v>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr">
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
         <is>
           <t>MDM2</t>
         </is>
@@ -1257,18 +1518,28 @@
         <v>1.99916691160039e-05</v>
       </c>
       <c r="F21" t="n">
+        <v>3.480031290563641e-05</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-1.278358846210356</v>
+      </c>
+      <c r="H21" t="n">
         <v>-0.8607203084848024</v>
       </c>
-      <c r="G21" t="n">
+      <c r="I21" t="n">
         <v>3.187627291507162e-05</v>
       </c>
-      <c r="H21" t="n">
+      <c r="J21" t="n">
+        <v>3.995159538688976e-05</v>
+      </c>
+      <c r="K21" t="n">
         <v>21</v>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr">
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
         <is>
           <t>MDM2</t>
         </is>
@@ -1295,18 +1566,28 @@
         <v>0.0004429851570295</v>
       </c>
       <c r="F22" t="n">
+        <v>0.0006034870255184</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-1.612606018434213</v>
+      </c>
+      <c r="H22" t="n">
         <v>-0.8385685386803599</v>
       </c>
-      <c r="G22" t="n">
+      <c r="I22" t="n">
         <v>0.0002561863437775</v>
       </c>
-      <c r="H22" t="n">
+      <c r="J22" t="n">
+        <v>0.0002833119566480588</v>
+      </c>
+      <c r="K22" t="n">
         <v>11</v>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr">
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
         <is>
           <t>NHLRC2</t>
         </is>
@@ -1333,18 +1614,28 @@
         <v>6.625351181132343e-17</v>
       </c>
       <c r="F23" t="n">
+        <v>4.448450078760288e-16</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-1.200210115640962</v>
+      </c>
+      <c r="H23" t="n">
         <v>-0.7854717076335129</v>
       </c>
-      <c r="G23" t="n">
+      <c r="I23" t="n">
         <v>4.915581987022988e-09</v>
       </c>
-      <c r="H23" t="n">
+      <c r="J23" t="n">
+        <v>8.885859745772323e-09</v>
+      </c>
+      <c r="K23" t="n">
         <v>68</v>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr">
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
         <is>
           <t>MDM2</t>
         </is>
@@ -1371,24 +1662,36 @@
         <v>1.441800374548279e-28</v>
       </c>
       <c r="F24" t="n">
+        <v>1.232083956432165e-27</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-1.110319560589528</v>
+      </c>
+      <c r="H24" t="n">
         <v>-0.8134129057753131</v>
       </c>
-      <c r="G24" t="n">
+      <c r="I24" t="n">
         <v>2.394191494511532e-41</v>
       </c>
-      <c r="H24" t="n">
+      <c r="J24" t="n">
+        <v>2.250540004840841e-39</v>
+      </c>
+      <c r="K24" t="n">
         <v>94</v>
       </c>
-      <c r="I24" t="n">
+      <c r="L24" t="n">
         <v>41</v>
       </c>
-      <c r="J24" t="n">
+      <c r="M24" t="n">
         <v>-0.6818914372162184</v>
       </c>
-      <c r="K24" t="n">
+      <c r="N24" t="n">
         <v>2.931096078334864e-12</v>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="O24" t="n">
+        <v>2.286254941101194e-11</v>
+      </c>
+      <c r="P24" t="inlineStr">
         <is>
           <t>ATP1B3</t>
         </is>
@@ -1415,24 +1718,36 @@
         <v>0.0212950430011134</v>
       </c>
       <c r="F25" t="n">
+        <v>0.0238301671679126</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-1.257657148122667</v>
+      </c>
+      <c r="H25" t="n">
         <v>-0.8174648918739086</v>
       </c>
-      <c r="G25" t="n">
+      <c r="I25" t="n">
         <v>1.120861106936203e-10</v>
       </c>
-      <c r="H25" t="n">
+      <c r="J25" t="n">
+        <v>2.569779123219588e-10</v>
+      </c>
+      <c r="K25" t="n">
         <v>42</v>
       </c>
-      <c r="I25" t="n">
+      <c r="L25" t="n">
         <v>41</v>
       </c>
-      <c r="J25" t="n">
+      <c r="M25" t="n">
         <v>-0.7743994149871708</v>
       </c>
-      <c r="K25" t="n">
+      <c r="N25" t="n">
         <v>6.563800164033292e-06</v>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="O25" t="n">
+        <v>1.163582756351356e-05</v>
+      </c>
+      <c r="P25" t="inlineStr">
         <is>
           <t>UMPS</t>
         </is>
@@ -1459,20 +1774,30 @@
         <v>0.0353499600566551</v>
       </c>
       <c r="F26" t="n">
+        <v>0.0381942097163859</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-1.437407598292096</v>
+      </c>
+      <c r="H26" t="n">
         <v>-0.7922003368754144</v>
       </c>
-      <c r="G26" t="n">
+      <c r="I26" t="n">
         <v>0.0003859202487365</v>
       </c>
-      <c r="H26" t="n">
+      <c r="J26" t="n">
+        <v>0.0004055298096389583</v>
+      </c>
+      <c r="K26" t="n">
         <v>7</v>
       </c>
-      <c r="I26" t="n">
+      <c r="L26" t="n">
         <v>2</v>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr">
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
         <is>
           <t>DCAF7</t>
         </is>
@@ -1499,24 +1824,36 @@
         <v>9.745357731664092e-05</v>
       </c>
       <c r="F27" t="n">
+        <v>0.0001477521978671</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-1.082122273813447</v>
+      </c>
+      <c r="H27" t="n">
         <v>-0.7857212986366928</v>
       </c>
-      <c r="G27" t="n">
+      <c r="I27" t="n">
         <v>1.985738654165092e-32</v>
       </c>
-      <c r="H27" t="n">
+      <c r="J27" t="n">
+        <v>4.666485837287967e-31</v>
+      </c>
+      <c r="K27" t="n">
         <v>94</v>
       </c>
-      <c r="I27" t="n">
+      <c r="L27" t="n">
         <v>41</v>
       </c>
-      <c r="J27" t="n">
+      <c r="M27" t="n">
         <v>-0.4595398417515101</v>
       </c>
-      <c r="K27" t="n">
+      <c r="N27" t="n">
         <v>8.034058362534247e-06</v>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="O27" t="n">
+        <v>1.362296852777546e-05</v>
+      </c>
+      <c r="P27" t="inlineStr">
         <is>
           <t>NAMPT</t>
         </is>
@@ -1543,18 +1880,28 @@
         <v>1.630459465092921e-13</v>
       </c>
       <c r="F28" t="n">
+        <v>6.663616944292809e-13</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-1.522591615377213</v>
+      </c>
+      <c r="H28" t="n">
         <v>-0.7841506114188979</v>
       </c>
-      <c r="G28" t="n">
-        <v>3.992209328978555e-11</v>
-      </c>
-      <c r="H28" t="n">
+      <c r="I28" t="n">
+        <v>3.992209328978554e-11</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1.042410213677734e-10</v>
+      </c>
+      <c r="K28" t="n">
         <v>63</v>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr">
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
         <is>
           <t>SNAP23</t>
         </is>
@@ -1581,24 +1928,36 @@
         <v>7.572587350113489e-09</v>
       </c>
       <c r="F29" t="n">
+        <v>2.296203906163445e-08</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-1.196063514301491</v>
+      </c>
+      <c r="H29" t="n">
         <v>-0.7737913303898769</v>
       </c>
-      <c r="G29" t="n">
+      <c r="I29" t="n">
         <v>4.437835256957793e-29</v>
       </c>
-      <c r="H29" t="n">
+      <c r="J29" t="n">
+        <v>5.214456426925407e-28</v>
+      </c>
+      <c r="K29" t="n">
         <v>94</v>
       </c>
-      <c r="I29" t="n">
+      <c r="L29" t="n">
         <v>41</v>
       </c>
-      <c r="J29" t="n">
+      <c r="M29" t="n">
         <v>-0.721043490182573</v>
       </c>
-      <c r="K29" t="n">
+      <c r="N29" t="n">
         <v>3.10207164675976e-09</v>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="O29" t="n">
+        <v>9.30621494027928e-09</v>
+      </c>
+      <c r="P29" t="inlineStr">
         <is>
           <t>UMPS</t>
         </is>
@@ -1625,18 +1984,28 @@
         <v>4.510072204204106e-07</v>
       </c>
       <c r="F30" t="n">
+        <v>1.0340165541346e-06</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-1.461931445337405</v>
+      </c>
+      <c r="H30" t="n">
         <v>-0.7629604440977227</v>
       </c>
-      <c r="G30" t="n">
+      <c r="I30" t="n">
         <v>4.726965449118245e-05</v>
       </c>
-      <c r="H30" t="n">
+      <c r="J30" t="n">
+        <v>5.77058119762487e-05</v>
+      </c>
+      <c r="K30" t="n">
         <v>34</v>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
         <is>
           <t>SEPHS2</t>
         </is>
@@ -1663,24 +2032,36 @@
         <v>5.00326172621582e-05</v>
       </c>
       <c r="F31" t="n">
+        <v>8.108734521798054e-05</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-1.414330407664655</v>
+      </c>
+      <c r="H31" t="n">
         <v>-0.7533715636271214</v>
       </c>
-      <c r="G31" t="n">
+      <c r="I31" t="n">
         <v>9.583404147016244e-23</v>
       </c>
-      <c r="H31" t="n">
+      <c r="J31" t="n">
+        <v>5.299058763644276e-22</v>
+      </c>
+      <c r="K31" t="n">
         <v>94</v>
       </c>
-      <c r="I31" t="n">
+      <c r="L31" t="n">
         <v>41</v>
       </c>
-      <c r="J31" t="n">
+      <c r="M31" t="n">
         <v>-0.4845765637944574</v>
       </c>
-      <c r="K31" t="n">
+      <c r="N31" t="n">
         <v>6.917305069341635e-05</v>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="O31" t="n">
+        <v>9.63481777515442e-05</v>
+      </c>
+      <c r="P31" t="inlineStr">
         <is>
           <t>SEPHS2</t>
         </is>
@@ -1707,18 +2088,28 @@
         <v>2.893712982107823e-15</v>
       </c>
       <c r="F32" t="n">
+        <v>1.564031353607828e-14</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-1.234013429452743</v>
+      </c>
+      <c r="H32" t="n">
         <v>-0.7640065570745299</v>
       </c>
-      <c r="G32" t="n">
+      <c r="I32" t="n">
         <v>2.19909435982719e-14</v>
       </c>
-      <c r="H32" t="n">
+      <c r="J32" t="n">
+        <v>7.950571916298303e-14</v>
+      </c>
+      <c r="K32" t="n">
         <v>68</v>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -1745,24 +2136,36 @@
         <v>0.0001339470885691</v>
       </c>
       <c r="F33" t="n">
+        <v>0.0001967347863358</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-1.575504219990485</v>
+      </c>
+      <c r="H33" t="n">
         <v>-0.7419609977589287</v>
       </c>
-      <c r="G33" t="n">
+      <c r="I33" t="n">
         <v>5.825276582270477e-26</v>
       </c>
-      <c r="H33" t="n">
+      <c r="J33" t="n">
+        <v>4.56313332277854e-25</v>
+      </c>
+      <c r="K33" t="n">
         <v>94</v>
       </c>
-      <c r="I33" t="n">
+      <c r="L33" t="n">
         <v>41</v>
       </c>
-      <c r="J33" t="n">
+      <c r="M33" t="n">
         <v>-0.673275388547977</v>
       </c>
-      <c r="K33" t="n">
+      <c r="N33" t="n">
         <v>3.885254537012033e-06</v>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="O33" t="n">
+        <v>7.215472711593775e-06</v>
+      </c>
+      <c r="P33" t="inlineStr">
         <is>
           <t>TFRC</t>
         </is>
@@ -1789,24 +2192,36 @@
         <v>0.0135991678847403</v>
       </c>
       <c r="F34" t="n">
+        <v>0.0157817503847603</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-1.056576298494927</v>
+      </c>
+      <c r="H34" t="n">
         <v>-0.7472285574080981</v>
       </c>
-      <c r="G34" t="n">
+      <c r="I34" t="n">
         <v>2.538819690216238e-15</v>
       </c>
-      <c r="H34" t="n">
+      <c r="J34" t="n">
+        <v>9.545962035213054e-15</v>
+      </c>
+      <c r="K34" t="n">
         <v>42</v>
       </c>
-      <c r="I34" t="n">
+      <c r="L34" t="n">
         <v>41</v>
       </c>
-      <c r="J34" t="n">
+      <c r="M34" t="n">
         <v>-0.4253291821174721</v>
       </c>
-      <c r="K34" t="n">
+      <c r="N34" t="n">
         <v>0.0002415525138377</v>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="O34" t="n">
+        <v>0.00031401826798901</v>
+      </c>
+      <c r="P34" t="inlineStr">
         <is>
           <t>NAMPT</t>
         </is>
@@ -1833,24 +2248,36 @@
         <v>2.759659594195708e-08</v>
       </c>
       <c r="F35" t="n">
+        <v>7.629647113364603e-08</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-1.128976862422515</v>
+      </c>
+      <c r="H35" t="n">
         <v>-0.7341203191826722</v>
       </c>
-      <c r="G35" t="n">
+      <c r="I35" t="n">
         <v>1.05618295388561e-29</v>
       </c>
-      <c r="H35" t="n">
+      <c r="J35" t="n">
+        <v>1.418302823789248e-28</v>
+      </c>
+      <c r="K35" t="n">
         <v>94</v>
       </c>
-      <c r="I35" t="n">
+      <c r="L35" t="n">
         <v>41</v>
       </c>
-      <c r="J35" t="n">
+      <c r="M35" t="n">
         <v>-0.586529726825697</v>
       </c>
-      <c r="K35" t="n">
+      <c r="N35" t="n">
         <v>1.092546182614044e-09</v>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="O35" t="n">
+        <v>3.873572829267974e-09</v>
+      </c>
+      <c r="P35" t="inlineStr">
         <is>
           <t>SDHB</t>
         </is>
@@ -1877,24 +2304,36 @@
         <v>0.0888406419230869</v>
       </c>
       <c r="F36" t="n">
+        <v>0.09383168922213669</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-1.699645549757265</v>
+      </c>
+      <c r="H36" t="n">
         <v>-0.7371457091738305</v>
       </c>
-      <c r="G36" t="n">
+      <c r="I36" t="n">
         <v>4.488076668414864e-11</v>
       </c>
-      <c r="H36" t="n">
+      <c r="J36" t="n">
+        <v>1.140214072516209e-10</v>
+      </c>
+      <c r="K36" t="n">
         <v>42</v>
       </c>
-      <c r="I36" t="n">
+      <c r="L36" t="n">
         <v>41</v>
       </c>
-      <c r="J36" t="n">
+      <c r="M36" t="n">
         <v>-0.5084031144778887</v>
       </c>
-      <c r="K36" t="n">
+      <c r="N36" t="n">
         <v>0.0002760060416073</v>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="O36" t="n">
+        <v>0.0003363823632088969</v>
+      </c>
+      <c r="P36" t="inlineStr">
         <is>
           <t>ADSL</t>
         </is>
@@ -1921,18 +2360,28 @@
         <v>3.83348282584508e-05</v>
       </c>
       <c r="F37" t="n">
+        <v>6.321883958411185e-05</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-1.796984303523731</v>
+      </c>
+      <c r="H37" t="n">
         <v>-0.7513597838953947</v>
       </c>
-      <c r="G37" t="n">
+      <c r="I37" t="n">
         <v>1.28759012579612e-07</v>
       </c>
-      <c r="H37" t="n">
+      <c r="J37" t="n">
+        <v>2.051414776692123e-07</v>
+      </c>
+      <c r="K37" t="n">
         <v>68</v>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr">
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
         <is>
           <t>CCND1</t>
         </is>
@@ -1959,20 +2408,30 @@
         <v>0.0148884280757132</v>
       </c>
       <c r="F38" t="n">
+        <v>0.0170672224282565</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-1.514616136205607</v>
+      </c>
+      <c r="H38" t="n">
         <v>-0.7216669481620047</v>
       </c>
-      <c r="G38" t="n">
+      <c r="I38" t="n">
         <v>0.0004035256005726</v>
       </c>
-      <c r="H38" t="n">
+      <c r="J38" t="n">
+        <v>0.0004122978962372218</v>
+      </c>
+      <c r="K38" t="n">
         <v>10</v>
       </c>
-      <c r="I38" t="n">
+      <c r="L38" t="n">
         <v>7</v>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr">
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
         <is>
           <t>SUMO2</t>
         </is>
@@ -1999,24 +2458,36 @@
         <v>0.0292194528351796</v>
       </c>
       <c r="F39" t="n">
+        <v>0.0323132772530221</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-1.63442958182128</v>
+      </c>
+      <c r="H39" t="n">
         <v>-0.717347388258246</v>
       </c>
-      <c r="G39" t="n">
+      <c r="I39" t="n">
         <v>4.74666416426053e-17</v>
       </c>
-      <c r="H39" t="n">
+      <c r="J39" t="n">
+        <v>1.859110131002041e-16</v>
+      </c>
+      <c r="K39" t="n">
         <v>94</v>
       </c>
-      <c r="I39" t="n">
+      <c r="L39" t="n">
         <v>41</v>
       </c>
-      <c r="J39" t="n">
+      <c r="M39" t="n">
         <v>-0.4298591836647585</v>
       </c>
-      <c r="K39" t="n">
+      <c r="N39" t="n">
         <v>0.0029038371528668</v>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="O39" t="n">
+        <v>0.003145823582272367</v>
+      </c>
+      <c r="P39" t="inlineStr">
         <is>
           <t>CDAN1</t>
         </is>
@@ -2043,24 +2514,36 @@
         <v>2.090280984449076e-19</v>
       </c>
       <c r="F40" t="n">
+        <v>1.637386771151776e-18</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-1.004941145021997</v>
+      </c>
+      <c r="H40" t="n">
         <v>-0.7138127847710718</v>
       </c>
-      <c r="G40" t="n">
+      <c r="I40" t="n">
         <v>8.598963279462991e-33</v>
       </c>
-      <c r="H40" t="n">
+      <c r="J40" t="n">
+        <v>2.694341827565071e-31</v>
+      </c>
+      <c r="K40" t="n">
         <v>94</v>
       </c>
-      <c r="I40" t="n">
+      <c r="L40" t="n">
         <v>41</v>
       </c>
-      <c r="J40" t="n">
+      <c r="M40" t="n">
         <v>-0.576014333987656</v>
       </c>
-      <c r="K40" t="n">
+      <c r="N40" t="n">
         <v>7.085328533664828e-11</v>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="O40" t="n">
+        <v>3.947540183041832e-10</v>
+      </c>
+      <c r="P40" t="inlineStr">
         <is>
           <t>EP300</t>
         </is>
@@ -2087,18 +2570,28 @@
         <v>3.592411582983894e-11</v>
       </c>
       <c r="F41" t="n">
+        <v>1.298794956924946e-10</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-1.673854449943091</v>
+      </c>
+      <c r="H41" t="n">
         <v>-0.7087627694107538</v>
       </c>
-      <c r="G41" t="n">
+      <c r="I41" t="n">
         <v>1.453637991757867e-10</v>
       </c>
-      <c r="H41" t="n">
+      <c r="J41" t="n">
+        <v>3.253380267267608e-10</v>
+      </c>
+      <c r="K41" t="n">
         <v>63</v>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
         <is>
           <t>BCL2L1</t>
         </is>
@@ -2125,18 +2618,28 @@
         <v>7.312073568677205e-19</v>
       </c>
       <c r="F42" t="n">
+        <v>5.28719165735121e-18</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-1.211311977116099</v>
+      </c>
+      <c r="H42" t="n">
         <v>-0.7085547354966818</v>
       </c>
-      <c r="G42" t="n">
+      <c r="I42" t="n">
         <v>3.728717773096875e-14</v>
       </c>
-      <c r="H42" t="n">
+      <c r="J42" t="n">
+        <v>1.298146187670764e-13</v>
+      </c>
+      <c r="K42" t="n">
         <v>63</v>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
         <is>
           <t>KRAS</t>
         </is>
@@ -2163,18 +2666,28 @@
         <v>1.461590086948102e-08</v>
       </c>
       <c r="F43" t="n">
+        <v>4.163317217367322e-08</v>
+      </c>
+      <c r="G43" t="n">
+        <v>-1.011961766589184</v>
+      </c>
+      <c r="H43" t="n">
         <v>-0.7069344954689746</v>
       </c>
-      <c r="G43" t="n">
+      <c r="I43" t="n">
         <v>5.428057264751609e-05</v>
       </c>
-      <c r="H43" t="n">
+      <c r="J43" t="n">
+        <v>6.541504908803222e-05</v>
+      </c>
+      <c r="K43" t="n">
         <v>10</v>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
         <is>
           <t>SOX10</t>
         </is>
@@ -2201,24 +2714,36 @@
         <v>0.0009193810892928</v>
       </c>
       <c r="F44" t="n">
+        <v>0.0012172087661059</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-1.624021565456589</v>
+      </c>
+      <c r="H44" t="n">
         <v>-0.7043483026148512</v>
       </c>
-      <c r="G44" t="n">
+      <c r="I44" t="n">
         <v>7.545571295499275e-23</v>
       </c>
-      <c r="H44" t="n">
+      <c r="J44" t="n">
+        <v>4.433023136105824e-22</v>
+      </c>
+      <c r="K44" t="n">
         <v>94</v>
       </c>
-      <c r="I44" t="n">
+      <c r="L44" t="n">
         <v>41</v>
       </c>
-      <c r="J44" t="n">
+      <c r="M44" t="n">
         <v>-0.4376418542348637</v>
       </c>
-      <c r="K44" t="n">
+      <c r="N44" t="n">
         <v>1.259831285977681e-05</v>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="O44" t="n">
+        <v>1.889746928966521e-05</v>
+      </c>
+      <c r="P44" t="inlineStr">
         <is>
           <t>ADSL</t>
         </is>
@@ -2245,18 +2770,28 @@
         <v>0.0001449830829607</v>
       </c>
       <c r="F45" t="n">
+        <v>0.0002096678430508</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-1.446877134048081</v>
+      </c>
+      <c r="H45" t="n">
         <v>-0.6968741219393133</v>
       </c>
-      <c r="G45" t="n">
+      <c r="I45" t="n">
         <v>4.600497157632777e-05</v>
       </c>
-      <c r="H45" t="n">
+      <c r="J45" t="n">
+        <v>5.690088589703698e-05</v>
+      </c>
+      <c r="K45" t="n">
         <v>21</v>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr">
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
         <is>
           <t>SNAP23</t>
         </is>
@@ -2283,18 +2818,28 @@
         <v>3.727226775396882e-08</v>
       </c>
       <c r="F46" t="n">
+        <v>1.00102661967802e-07</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-1.656857628342071</v>
+      </c>
+      <c r="H46" t="n">
         <v>-0.6867075681179416</v>
       </c>
-      <c r="G46" t="n">
+      <c r="I46" t="n">
         <v>5.318266714980121e-08</v>
       </c>
-      <c r="H46" t="n">
+      <c r="J46" t="n">
+        <v>9.089401294693299e-08</v>
+      </c>
+      <c r="K46" t="n">
         <v>63</v>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr">
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr">
         <is>
           <t>SCAP</t>
         </is>
@@ -2321,20 +2866,30 @@
         <v>0.002750289889322</v>
       </c>
       <c r="F47" t="n">
+        <v>0.0034936114810306</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-2.431461893651065</v>
+      </c>
+      <c r="H47" t="n">
         <v>-0.6764773540686089</v>
       </c>
-      <c r="G47" t="n">
+      <c r="I47" t="n">
         <v>5.756471953078053e-06</v>
       </c>
-      <c r="H47" t="n">
+      <c r="J47" t="n">
+        <v>7.730119479847672e-06</v>
+      </c>
+      <c r="K47" t="n">
         <v>10</v>
       </c>
-      <c r="I47" t="n">
+      <c r="L47" t="n">
         <v>9</v>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr">
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr">
         <is>
           <t>WDR36</t>
         </is>
@@ -2361,18 +2916,28 @@
         <v>8.535856631369382e-07</v>
       </c>
       <c r="F48" t="n">
+        <v>1.865977961276098e-06</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-1.137284631353363</v>
+      </c>
+      <c r="H48" t="n">
         <v>-0.6755232533141455</v>
       </c>
-      <c r="G48" t="n">
+      <c r="I48" t="n">
         <v>7.525447425741933e-05</v>
       </c>
-      <c r="H48" t="n">
+      <c r="J48" t="n">
+        <v>8.95432984835116e-05</v>
+      </c>
+      <c r="K48" t="n">
         <v>63</v>
       </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr">
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr">
         <is>
           <t>FAM50A</t>
         </is>
@@ -2399,24 +2964,36 @@
         <v>2.74261262861531e-07</v>
       </c>
       <c r="F49" t="n">
+        <v>6.445139677245978e-07</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-1.084876209676264</v>
+      </c>
+      <c r="H49" t="n">
         <v>-0.6708233312019126</v>
       </c>
-      <c r="G49" t="n">
+      <c r="I49" t="n">
         <v>2.712005242470748e-28</v>
       </c>
-      <c r="H49" t="n">
+      <c r="J49" t="n">
+        <v>2.549284927922504e-27</v>
+      </c>
+      <c r="K49" t="n">
         <v>94</v>
       </c>
-      <c r="I49" t="n">
+      <c r="L49" t="n">
         <v>41</v>
       </c>
-      <c r="J49" t="n">
+      <c r="M49" t="n">
         <v>-0.4216744548314787</v>
       </c>
-      <c r="K49" t="n">
+      <c r="N49" t="n">
         <v>1.040143861038079e-05</v>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="O49" t="n">
+        <v>1.690233774186878e-05</v>
+      </c>
+      <c r="P49" t="inlineStr">
         <is>
           <t>FPGS</t>
         </is>
@@ -2443,24 +3020,36 @@
         <v>4.398029969151889e-10</v>
       </c>
       <c r="F50" t="n">
+        <v>1.531165989260287e-09</v>
+      </c>
+      <c r="G50" t="n">
+        <v>-1.098108830659307</v>
+      </c>
+      <c r="H50" t="n">
         <v>-0.6671348838654333</v>
       </c>
-      <c r="G50" t="n">
+      <c r="I50" t="n">
         <v>1.795252001275173e-31</v>
       </c>
-      <c r="H50" t="n">
+      <c r="J50" t="n">
+        <v>3.375073762397325e-30</v>
+      </c>
+      <c r="K50" t="n">
         <v>94</v>
       </c>
-      <c r="I50" t="n">
+      <c r="L50" t="n">
         <v>41</v>
       </c>
-      <c r="J50" t="n">
+      <c r="M50" t="n">
         <v>-0.4925197507548559</v>
       </c>
-      <c r="K50" t="n">
+      <c r="N50" t="n">
         <v>4.712803000355117e-08</v>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="O50" t="n">
+        <v>1.110062280262243e-07</v>
+      </c>
+      <c r="P50" t="inlineStr">
         <is>
           <t>PAICS</t>
         </is>
@@ -2487,24 +3076,36 @@
         <v>0.0165864233862047</v>
       </c>
       <c r="F51" t="n">
+        <v>0.0187846240759426</v>
+      </c>
+      <c r="G51" t="n">
+        <v>-1.194925027264708</v>
+      </c>
+      <c r="H51" t="n">
         <v>-0.6955237028569836</v>
       </c>
-      <c r="G51" t="n">
+      <c r="I51" t="n">
         <v>0.0001481671849292</v>
       </c>
-      <c r="H51" t="n">
+      <c r="J51" t="n">
+        <v>0.000171947103498084</v>
+      </c>
+      <c r="K51" t="n">
         <v>42</v>
       </c>
-      <c r="I51" t="n">
+      <c r="L51" t="n">
         <v>41</v>
       </c>
-      <c r="J51" t="n">
+      <c r="M51" t="n">
         <v>-0.7142326805938296</v>
       </c>
-      <c r="K51" t="n">
+      <c r="N51" t="n">
         <v>0.0064284212081502</v>
       </c>
-      <c r="L51" t="inlineStr">
+      <c r="O51" t="n">
+        <v>0.006775903435617779</v>
+      </c>
+      <c r="P51" t="inlineStr">
         <is>
           <t>TYMS</t>
         </is>
@@ -2531,18 +3132,28 @@
         <v>1.214124744033309e-06</v>
       </c>
       <c r="F52" t="n">
+        <v>2.428249488066618e-06</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-1.134767216750626</v>
+      </c>
+      <c r="H52" t="n">
         <v>-0.6595481102626115</v>
       </c>
-      <c r="G52" t="n">
+      <c r="I52" t="n">
         <v>2.512633176712835e-08</v>
       </c>
-      <c r="H52" t="n">
+      <c r="J52" t="n">
+        <v>4.37384293724086e-08</v>
+      </c>
+      <c r="K52" t="n">
         <v>49</v>
       </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -2569,24 +3180,36 @@
         <v>0.0076473869843637</v>
       </c>
       <c r="F53" t="n">
+        <v>0.009335771123768599</v>
+      </c>
+      <c r="G53" t="n">
+        <v>-1.108807893958623</v>
+      </c>
+      <c r="H53" t="n">
         <v>-0.655227558198187</v>
       </c>
-      <c r="G53" t="n">
+      <c r="I53" t="n">
         <v>1.921001848956053e-08</v>
       </c>
-      <c r="H53" t="n">
+      <c r="J53" t="n">
+        <v>3.407059883054132e-08</v>
+      </c>
+      <c r="K53" t="n">
         <v>94</v>
       </c>
-      <c r="I53" t="n">
+      <c r="L53" t="n">
         <v>41</v>
       </c>
-      <c r="J53" t="n">
+      <c r="M53" t="n">
         <v>-0.6702686243994869</v>
       </c>
-      <c r="K53" t="n">
+      <c r="N53" t="n">
         <v>0.0004376104608551</v>
       </c>
-      <c r="L53" t="inlineStr">
+      <c r="O53" t="n">
+        <v>0.000517175999192391</v>
+      </c>
+      <c r="P53" t="inlineStr">
         <is>
           <t>FAM50A</t>
         </is>
@@ -2613,18 +3236,28 @@
         <v>0.0063423310909463</v>
       </c>
       <c r="F54" t="n">
+        <v>0.007844462138801999</v>
+      </c>
+      <c r="G54" t="n">
+        <v>-1.656290751490781</v>
+      </c>
+      <c r="H54" t="n">
         <v>-0.6374202364926882</v>
       </c>
-      <c r="G54" t="n">
+      <c r="I54" t="n">
         <v>0.0001786778067235</v>
       </c>
-      <c r="H54" t="n">
+      <c r="J54" t="n">
+        <v>0.0001999489741905833</v>
+      </c>
+      <c r="K54" t="n">
         <v>25</v>
       </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr">
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr">
         <is>
           <t>GRB2</t>
         </is>
@@ -2651,24 +3284,36 @@
         <v>0.0014621264034239</v>
       </c>
       <c r="F55" t="n">
+        <v>0.0019088872489145</v>
+      </c>
+      <c r="G55" t="n">
+        <v>-1.861901919664883</v>
+      </c>
+      <c r="H55" t="n">
         <v>-0.6456273309877603</v>
       </c>
-      <c r="G55" t="n">
+      <c r="I55" t="n">
         <v>1.357147635527964e-09</v>
       </c>
-      <c r="H55" t="n">
+      <c r="J55" t="n">
+        <v>2.657747452908929e-09</v>
+      </c>
+      <c r="K55" t="n">
         <v>94</v>
       </c>
-      <c r="I55" t="n">
+      <c r="L55" t="n">
         <v>41</v>
       </c>
-      <c r="J55" t="n">
+      <c r="M55" t="n">
         <v>-0.6550159891805287</v>
       </c>
-      <c r="K55" t="n">
+      <c r="N55" t="n">
         <v>0.0002730818864878</v>
       </c>
-      <c r="L55" t="inlineStr">
+      <c r="O55" t="n">
+        <v>0.0003363823632088969</v>
+      </c>
+      <c r="P55" t="inlineStr">
         <is>
           <t>DNAJC9</t>
         </is>
@@ -2695,24 +3340,36 @@
         <v>0.0058440679493856</v>
       </c>
       <c r="F56" t="n">
+        <v>0.0073245651632299</v>
+      </c>
+      <c r="G56" t="n">
+        <v>-1.283242500875942</v>
+      </c>
+      <c r="H56" t="n">
         <v>-0.649236875917413</v>
       </c>
-      <c r="G56" t="n">
+      <c r="I56" t="n">
         <v>4.9029989231975e-11</v>
       </c>
-      <c r="H56" t="n">
+      <c r="J56" t="n">
+        <v>1.212847102054119e-10</v>
+      </c>
+      <c r="K56" t="n">
         <v>42</v>
       </c>
-      <c r="I56" t="n">
+      <c r="L56" t="n">
         <v>41</v>
       </c>
-      <c r="J56" t="n">
+      <c r="M56" t="n">
         <v>-0.5370362933349632</v>
       </c>
-      <c r="K56" t="n">
+      <c r="N56" t="n">
         <v>1.250055161433351e-05</v>
       </c>
-      <c r="L56" t="inlineStr">
+      <c r="O56" t="n">
+        <v>1.889746928966521e-05</v>
+      </c>
+      <c r="P56" t="inlineStr">
         <is>
           <t>TRPM7</t>
         </is>
@@ -2739,18 +3396,28 @@
         <v>5.375366681084805e-12</v>
       </c>
       <c r="F57" t="n">
+        <v>2.105351950091549e-11</v>
+      </c>
+      <c r="G57" t="n">
+        <v>-1.811098652249668</v>
+      </c>
+      <c r="H57" t="n">
         <v>-0.6286606562208354</v>
       </c>
-      <c r="G57" t="n">
+      <c r="I57" t="n">
         <v>4.834763208780085e-12</v>
       </c>
-      <c r="H57" t="n">
+      <c r="J57" t="n">
+        <v>1.336669828309788e-11</v>
+      </c>
+      <c r="K57" t="n">
         <v>47</v>
       </c>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr">
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr">
         <is>
           <t>CHMP4B</t>
         </is>
@@ -2777,24 +3444,36 @@
         <v>1.162462502063463e-06</v>
       </c>
       <c r="F58" t="n">
+        <v>2.375466852042729e-06</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-1.219805078787887</v>
+      </c>
+      <c r="H58" t="n">
         <v>-0.6360650198377347</v>
       </c>
-      <c r="G58" t="n">
+      <c r="I58" t="n">
         <v>5.352577169744143e-21</v>
       </c>
-      <c r="H58" t="n">
+      <c r="J58" t="n">
+        <v>2.515711269779747e-20</v>
+      </c>
+      <c r="K58" t="n">
         <v>94</v>
       </c>
-      <c r="I58" t="n">
+      <c r="L58" t="n">
         <v>41</v>
       </c>
-      <c r="J58" t="n">
+      <c r="M58" t="n">
         <v>-0.6644835481967274</v>
       </c>
-      <c r="K58" t="n">
+      <c r="N58" t="n">
         <v>1.097346498744284e-10</v>
       </c>
-      <c r="L58" t="inlineStr">
+      <c r="O58" t="n">
+        <v>5.349564181378385e-10</v>
+      </c>
+      <c r="P58" t="inlineStr">
         <is>
           <t>CTPS1</t>
         </is>
@@ -2821,24 +3500,36 @@
         <v>7.080631664356068e-16</v>
       </c>
       <c r="F59" t="n">
+        <v>4.437195842996469e-15</v>
+      </c>
+      <c r="G59" t="n">
+        <v>-1.196017737896068</v>
+      </c>
+      <c r="H59" t="n">
         <v>-0.6282553320969391</v>
       </c>
-      <c r="G59" t="n">
+      <c r="I59" t="n">
         <v>3.854784429689131e-30</v>
       </c>
-      <c r="H59" t="n">
+      <c r="J59" t="n">
+        <v>6.039162273179638e-29</v>
+      </c>
+      <c r="K59" t="n">
         <v>94</v>
       </c>
-      <c r="I59" t="n">
+      <c r="L59" t="n">
         <v>41</v>
       </c>
-      <c r="J59" t="n">
+      <c r="M59" t="n">
         <v>-0.7508429907014329</v>
       </c>
-      <c r="K59" t="n">
+      <c r="N59" t="n">
         <v>2.129449692085123e-14</v>
       </c>
-      <c r="L59" t="inlineStr">
+      <c r="O59" t="n">
+        <v>7.18998652506705e-13</v>
+      </c>
+      <c r="P59" t="inlineStr">
         <is>
           <t>CFL1</t>
         </is>
@@ -2865,18 +3556,28 @@
         <v>1.592564136721469e-09</v>
       </c>
       <c r="F60" t="n">
+        <v>5.162104443166141e-09</v>
+      </c>
+      <c r="G60" t="n">
+        <v>-1.085801676852166</v>
+      </c>
+      <c r="H60" t="n">
         <v>-0.621127911654316</v>
       </c>
-      <c r="G60" t="n">
+      <c r="I60" t="n">
         <v>1.48616928243708e-11</v>
       </c>
-      <c r="H60" t="n">
+      <c r="J60" t="n">
+        <v>3.991426072831016e-11</v>
+      </c>
+      <c r="K60" t="n">
         <v>91</v>
       </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr">
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -2903,24 +3604,36 @@
         <v>0.030420349847232</v>
       </c>
       <c r="F61" t="n">
+        <v>0.033250149833021</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-1.505100079515383</v>
+      </c>
+      <c r="H61" t="n">
         <v>-0.6272267805769938</v>
       </c>
-      <c r="G61" t="n">
+      <c r="I61" t="n">
         <v>7.472616595858115e-11</v>
       </c>
-      <c r="H61" t="n">
+      <c r="J61" t="n">
+        <v>1.801092205155546e-10</v>
+      </c>
+      <c r="K61" t="n">
         <v>42</v>
       </c>
-      <c r="I61" t="n">
+      <c r="L61" t="n">
         <v>41</v>
       </c>
-      <c r="J61" t="n">
+      <c r="M61" t="n">
         <v>-0.5914172086955134</v>
       </c>
-      <c r="K61" t="n">
+      <c r="N61" t="n">
         <v>0.0002183921547255</v>
       </c>
-      <c r="L61" t="inlineStr">
+      <c r="O61" t="n">
+        <v>0.0002936997942860172</v>
+      </c>
+      <c r="P61" t="inlineStr">
         <is>
           <t>TFRC</t>
         </is>
@@ -2947,18 +3660,28 @@
         <v>0.0015322460691748</v>
       </c>
       <c r="F62" t="n">
+        <v>0.0019730291849648</v>
+      </c>
+      <c r="G62" t="n">
+        <v>-1.079861899639728</v>
+      </c>
+      <c r="H62" t="n">
         <v>-0.6064894498219039</v>
       </c>
-      <c r="G62" t="n">
+      <c r="I62" t="n">
         <v>0.0009634210920643</v>
       </c>
-      <c r="H62" t="n">
+      <c r="J62" t="n">
+        <v>0.0009634210920643</v>
+      </c>
+      <c r="K62" t="n">
         <v>34</v>
       </c>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr">
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr">
         <is>
           <t>FAM50A</t>
         </is>
@@ -2985,24 +3708,36 @@
         <v>0.7773861784358157</v>
       </c>
       <c r="F63" t="n">
+        <v>0.7773861784358157</v>
+      </c>
+      <c r="G63" t="n">
+        <v>-1.310266817725494</v>
+      </c>
+      <c r="H63" t="n">
         <v>-0.6167775413301757</v>
       </c>
-      <c r="G63" t="n">
+      <c r="I63" t="n">
         <v>6.956194496326791e-07</v>
       </c>
-      <c r="H63" t="n">
+      <c r="J63" t="n">
+        <v>1.00597274254572e-06</v>
+      </c>
+      <c r="K63" t="n">
         <v>42</v>
       </c>
-      <c r="I63" t="n">
+      <c r="L63" t="n">
         <v>41</v>
       </c>
-      <c r="J63" t="n">
+      <c r="M63" t="n">
         <v>-0.3650361080776294</v>
       </c>
-      <c r="K63" t="n">
+      <c r="N63" t="n">
         <v>0.0169685710870337</v>
       </c>
-      <c r="L63" t="inlineStr">
+      <c r="O63" t="n">
+        <v>0.01741511243142933</v>
+      </c>
+      <c r="P63" t="inlineStr">
         <is>
           <t>SEPHS2</t>
         </is>
@@ -3029,18 +3764,28 @@
         <v>0.0125803902232771</v>
       </c>
       <c r="F64" t="n">
+        <v>0.0147819585123505</v>
+      </c>
+      <c r="G64" t="n">
+        <v>-1.086130185369127</v>
+      </c>
+      <c r="H64" t="n">
         <v>-0.5916865997708414</v>
       </c>
-      <c r="G64" t="n">
+      <c r="I64" t="n">
         <v>0.0003925873689058</v>
       </c>
-      <c r="H64" t="n">
+      <c r="J64" t="n">
+        <v>0.0004055298096389583</v>
+      </c>
+      <c r="K64" t="n">
         <v>21</v>
       </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr">
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -3067,18 +3812,28 @@
         <v>0.0002463815997421</v>
       </c>
       <c r="F65" t="n">
+        <v>0.0003456697071008</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-1.408545036658453</v>
+      </c>
+      <c r="H65" t="n">
         <v>-0.5774407016587395</v>
       </c>
-      <c r="G65" t="n">
+      <c r="I65" t="n">
         <v>1.956853807214076e-07</v>
       </c>
-      <c r="H65" t="n">
+      <c r="J65" t="n">
+        <v>2.966842869001986e-07</v>
+      </c>
+      <c r="K65" t="n">
         <v>68</v>
       </c>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr">
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr">
         <is>
           <t>INTS6</t>
         </is>
@@ -3105,18 +3860,28 @@
         <v>0.0001249660657188</v>
       </c>
       <c r="F66" t="n">
+        <v>0.0001864573044058</v>
+      </c>
+      <c r="G66" t="n">
+        <v>-1.652638001425365</v>
+      </c>
+      <c r="H66" t="n">
         <v>-0.5883819733319164</v>
       </c>
-      <c r="G66" t="n">
+      <c r="I66" t="n">
         <v>0.0002980689475257</v>
       </c>
-      <c r="H66" t="n">
+      <c r="J66" t="n">
+        <v>0.0003220515065220207</v>
+      </c>
+      <c r="K66" t="n">
         <v>69</v>
       </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr">
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr">
         <is>
           <t>CCND1</t>
         </is>
@@ -3143,24 +3908,36 @@
         <v>9.41170290157365e-07</v>
       </c>
       <c r="F67" t="n">
+        <v>2.010681983518007e-06</v>
+      </c>
+      <c r="G67" t="n">
+        <v>-1.129221555732847</v>
+      </c>
+      <c r="H67" t="n">
         <v>-0.5885649499896715</v>
       </c>
-      <c r="G67" t="n">
+      <c r="I67" t="n">
         <v>2.717040561835115e-19</v>
       </c>
-      <c r="H67" t="n">
+      <c r="J67" t="n">
+        <v>1.110442664402178e-18</v>
+      </c>
+      <c r="K67" t="n">
         <v>94</v>
       </c>
-      <c r="I67" t="n">
+      <c r="L67" t="n">
         <v>41</v>
       </c>
-      <c r="J67" t="n">
+      <c r="M67" t="n">
         <v>-0.6945131202170721</v>
       </c>
-      <c r="K67" t="n">
+      <c r="N67" t="n">
         <v>6.866204754620908e-11</v>
       </c>
-      <c r="L67" t="inlineStr">
+      <c r="O67" t="n">
+        <v>3.947540183041832e-10</v>
+      </c>
+      <c r="P67" t="inlineStr">
         <is>
           <t>UROD</t>
         </is>
@@ -3187,18 +3964,28 @@
         <v>6.257121900727413e-09</v>
       </c>
       <c r="F68" t="n">
+        <v>1.960564862227923e-08</v>
+      </c>
+      <c r="G68" t="n">
+        <v>-1.563064365592713</v>
+      </c>
+      <c r="H68" t="n">
         <v>-0.5839010476423524</v>
       </c>
-      <c r="G68" t="n">
+      <c r="I68" t="n">
         <v>3.069318749913665e-13</v>
       </c>
-      <c r="H68" t="n">
+      <c r="J68" t="n">
+        <v>9.617198749729484e-13</v>
+      </c>
+      <c r="K68" t="n">
         <v>77</v>
       </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr">
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr">
         <is>
           <t>GRB2</t>
         </is>
@@ -3225,24 +4012,36 @@
         <v>0.1314110825595688</v>
       </c>
       <c r="F69" t="n">
+        <v>0.1372515751177718</v>
+      </c>
+      <c r="G69" t="n">
+        <v>-1.009147192525029</v>
+      </c>
+      <c r="H69" t="n">
         <v>-0.5942628025252563</v>
       </c>
-      <c r="G69" t="n">
+      <c r="I69" t="n">
         <v>3.426462089244155e-12</v>
       </c>
-      <c r="H69" t="n">
+      <c r="J69" t="n">
+        <v>1.006523238715471e-11</v>
+      </c>
+      <c r="K69" t="n">
         <v>42</v>
       </c>
-      <c r="I69" t="n">
+      <c r="L69" t="n">
         <v>41</v>
       </c>
-      <c r="J69" t="n">
+      <c r="M69" t="n">
         <v>-0.4594738773346523</v>
       </c>
-      <c r="K69" t="n">
+      <c r="N69" t="n">
         <v>9.229476573964988e-07</v>
       </c>
-      <c r="L69" t="inlineStr">
+      <c r="O69" t="n">
+        <v>1.799747931923173e-06</v>
+      </c>
+      <c r="P69" t="inlineStr">
         <is>
           <t>SDHB</t>
         </is>
@@ -3269,24 +4068,36 @@
         <v>7.295166160730784e-07</v>
       </c>
       <c r="F70" t="n">
+        <v>1.632727664544509e-06</v>
+      </c>
+      <c r="G70" t="n">
+        <v>-1.359704319580233</v>
+      </c>
+      <c r="H70" t="n">
         <v>-0.5906895447721376</v>
       </c>
-      <c r="G70" t="n">
+      <c r="I70" t="n">
         <v>1.561483691699727e-12</v>
       </c>
-      <c r="H70" t="n">
+      <c r="J70" t="n">
+        <v>4.734821516766915e-12</v>
+      </c>
+      <c r="K70" t="n">
         <v>42</v>
       </c>
-      <c r="I70" t="n">
+      <c r="L70" t="n">
         <v>41</v>
       </c>
-      <c r="J70" t="n">
+      <c r="M70" t="n">
         <v>-0.6704509625010068</v>
       </c>
-      <c r="K70" t="n">
+      <c r="N70" t="n">
         <v>3.581054951629473e-08</v>
       </c>
-      <c r="L70" t="inlineStr">
+      <c r="O70" t="n">
+        <v>9.310742874236628e-08</v>
+      </c>
+      <c r="P70" t="inlineStr">
         <is>
           <t>AP2S1</t>
         </is>
@@ -3313,18 +4124,28 @@
         <v>5.981291938388129e-05</v>
       </c>
       <c r="F71" t="n">
+        <v>9.370690703474736e-05</v>
+      </c>
+      <c r="G71" t="n">
+        <v>-1.564790426979868</v>
+      </c>
+      <c r="H71" t="n">
         <v>-0.5597986645385669</v>
       </c>
-      <c r="G71" t="n">
+      <c r="I71" t="n">
         <v>1.388112296327887e-06</v>
       </c>
-      <c r="H71" t="n">
+      <c r="J71" t="n">
+        <v>1.977008422042748e-06</v>
+      </c>
+      <c r="K71" t="n">
         <v>34</v>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr">
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
+      <c r="P71" t="inlineStr">
         <is>
           <t>GRB2</t>
         </is>
@@ -3351,18 +4172,28 @@
         <v>1.320554696871435e-07</v>
       </c>
       <c r="F72" t="n">
+        <v>3.354922743403105e-07</v>
+      </c>
+      <c r="G72" t="n">
+        <v>-1.763019369775018</v>
+      </c>
+      <c r="H72" t="n">
         <v>-0.5734873967234444</v>
       </c>
-      <c r="G72" t="n">
+      <c r="I72" t="n">
         <v>1.38561723036223e-07</v>
       </c>
-      <c r="H72" t="n">
+      <c r="J72" t="n">
+        <v>2.170800327567494e-07</v>
+      </c>
+      <c r="K72" t="n">
         <v>49</v>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr">
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr">
         <is>
           <t>CHMP4B</t>
         </is>
@@ -3389,18 +4220,28 @@
         <v>0.0122832924611463</v>
       </c>
       <c r="F73" t="n">
+        <v>0.0146155631816171</v>
+      </c>
+      <c r="G73" t="n">
+        <v>-1.630902550954251</v>
+      </c>
+      <c r="H73" t="n">
         <v>-0.5672009446450772</v>
       </c>
-      <c r="G73" t="n">
+      <c r="I73" t="n">
         <v>9.573614054035136e-05</v>
       </c>
-      <c r="H73" t="n">
+      <c r="J73" t="n">
+        <v>0.0001124899651349129</v>
+      </c>
+      <c r="K73" t="n">
         <v>48</v>
       </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr">
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr">
         <is>
           <t>CCND1</t>
         </is>
@@ -3427,24 +4268,36 @@
         <v>0.008052595716382401</v>
       </c>
       <c r="F74" t="n">
+        <v>0.0097044102223069</v>
+      </c>
+      <c r="G74" t="n">
+        <v>-1.180753668104172</v>
+      </c>
+      <c r="H74" t="n">
         <v>-0.568659414147102</v>
       </c>
-      <c r="G74" t="n">
+      <c r="I74" t="n">
         <v>2.236623580031438e-10</v>
       </c>
-      <c r="H74" t="n">
+      <c r="J74" t="n">
+        <v>4.889363174952446e-10</v>
+      </c>
+      <c r="K74" t="n">
         <v>42</v>
       </c>
-      <c r="I74" t="n">
+      <c r="L74" t="n">
         <v>41</v>
       </c>
-      <c r="J74" t="n">
+      <c r="M74" t="n">
         <v>-0.6252251687994282</v>
       </c>
-      <c r="K74" t="n">
+      <c r="N74" t="n">
         <v>1.862807931210987e-08</v>
       </c>
-      <c r="L74" t="inlineStr">
+      <c r="O74" t="n">
+        <v>5.189250665516321e-08</v>
+      </c>
+      <c r="P74" t="inlineStr">
         <is>
           <t>CTPS1</t>
         </is>
@@ -3471,18 +4324,28 @@
         <v>8.66467112002183e-09</v>
       </c>
       <c r="F75" t="n">
+        <v>2.545247141506413e-08</v>
+      </c>
+      <c r="G75" t="n">
+        <v>-1.307557453374142</v>
+      </c>
+      <c r="H75" t="n">
         <v>-0.5653455274197769</v>
       </c>
-      <c r="G75" t="n">
+      <c r="I75" t="n">
         <v>3.917403120301346e-07</v>
       </c>
-      <c r="H75" t="n">
+      <c r="J75" t="n">
+        <v>5.753685832942602e-07</v>
+      </c>
+      <c r="K75" t="n">
         <v>69</v>
       </c>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr">
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
+      <c r="P75" t="inlineStr">
         <is>
           <t>SNAP23</t>
         </is>
@@ -3509,24 +4372,36 @@
         <v>0.389179032142069</v>
       </c>
       <c r="F76" t="n">
+        <v>0.3976394458842879</v>
+      </c>
+      <c r="G76" t="n">
+        <v>-1.529616875876403</v>
+      </c>
+      <c r="H76" t="n">
         <v>-0.5719892820258186</v>
       </c>
-      <c r="G76" t="n">
+      <c r="I76" t="n">
         <v>4.682545553777284e-06</v>
       </c>
-      <c r="H76" t="n">
+      <c r="J76" t="n">
+        <v>6.379120029783546e-06</v>
+      </c>
+      <c r="K76" t="n">
         <v>42</v>
       </c>
-      <c r="I76" t="n">
+      <c r="L76" t="n">
         <v>41</v>
       </c>
-      <c r="J76" t="n">
+      <c r="M76" t="n">
         <v>-0.313987117065535</v>
       </c>
-      <c r="K76" t="n">
+      <c r="N76" t="n">
         <v>0.052648770197993</v>
       </c>
-      <c r="L76" t="inlineStr">
+      <c r="O76" t="n">
+        <v>0.052648770197993</v>
+      </c>
+      <c r="P76" t="inlineStr">
         <is>
           <t>CDAN1</t>
         </is>
@@ -3553,24 +4428,36 @@
         <v>0.1918507930290651</v>
       </c>
       <c r="F77" t="n">
+        <v>0.1981755444476057</v>
+      </c>
+      <c r="G77" t="n">
+        <v>-1.040453467812631</v>
+      </c>
+      <c r="H77" t="n">
         <v>-0.5749302366067428</v>
       </c>
-      <c r="G77" t="n">
+      <c r="I77" t="n">
         <v>0.0001707081891762</v>
       </c>
-      <c r="H77" t="n">
+      <c r="J77" t="n">
+        <v>0.0001933321660549735</v>
+      </c>
+      <c r="K77" t="n">
         <v>42</v>
       </c>
-      <c r="I77" t="n">
+      <c r="L77" t="n">
         <v>41</v>
       </c>
-      <c r="J77" t="n">
+      <c r="M77" t="n">
         <v>-0.5898299072848225</v>
       </c>
-      <c r="K77" t="n">
+      <c r="N77" t="n">
         <v>0.0017657027554503</v>
       </c>
-      <c r="L77" t="inlineStr">
+      <c r="O77" t="n">
+        <v>0.001967497356073191</v>
+      </c>
+      <c r="P77" t="inlineStr">
         <is>
           <t>FAM50A</t>
         </is>
@@ -3597,24 +4484,36 @@
         <v>2.142856641492325e-05</v>
       </c>
       <c r="F78" t="n">
+        <v>3.66233680545961e-05</v>
+      </c>
+      <c r="G78" t="n">
+        <v>-1.244820848235848</v>
+      </c>
+      <c r="H78" t="n">
         <v>-0.5732560602259542</v>
       </c>
-      <c r="G78" t="n">
+      <c r="I78" t="n">
         <v>2.869684589147233e-10</v>
       </c>
-      <c r="H78" t="n">
+      <c r="J78" t="n">
+        <v>6.130689804087269e-10</v>
+      </c>
+      <c r="K78" t="n">
         <v>42</v>
       </c>
-      <c r="I78" t="n">
+      <c r="L78" t="n">
         <v>41</v>
       </c>
-      <c r="J78" t="n">
+      <c r="M78" t="n">
         <v>-0.5787343392158727</v>
       </c>
-      <c r="K78" t="n">
+      <c r="N78" t="n">
         <v>8.661693539560024e-08</v>
       </c>
-      <c r="L78" t="inlineStr">
+      <c r="O78" t="n">
+        <v>1.876700266904672e-07</v>
+      </c>
+      <c r="P78" t="inlineStr">
         <is>
           <t>MED1</t>
         </is>
@@ -3641,24 +4540,36 @@
         <v>5.380048833393938e-05</v>
       </c>
       <c r="F79" t="n">
+        <v>8.571603226085258e-05</v>
+      </c>
+      <c r="G79" t="n">
+        <v>-1.280779954131551</v>
+      </c>
+      <c r="H79" t="n">
         <v>-0.5606742930512293</v>
       </c>
-      <c r="G79" t="n">
+      <c r="I79" t="n">
         <v>1.721007650944713e-19</v>
       </c>
-      <c r="H79" t="n">
+      <c r="J79" t="n">
+        <v>7.353396326763774e-19</v>
+      </c>
+      <c r="K79" t="n">
         <v>89</v>
       </c>
-      <c r="I79" t="n">
+      <c r="L79" t="n">
         <v>38</v>
       </c>
-      <c r="J79" t="n">
+      <c r="M79" t="n">
         <v>-0.3941146680757215</v>
       </c>
-      <c r="K79" t="n">
+      <c r="N79" t="n">
         <v>3.884982873798152e-05</v>
       </c>
-      <c r="L79" t="inlineStr">
+      <c r="O79" t="n">
+        <v>5.611641928819553e-05</v>
+      </c>
+      <c r="P79" t="inlineStr">
         <is>
           <t>DHFR</t>
         </is>
@@ -3685,18 +4596,28 @@
         <v>3.314403007253767e-15</v>
       </c>
       <c r="F80" t="n">
+        <v>1.639757277272916e-14</v>
+      </c>
+      <c r="G80" t="n">
+        <v>-1.252704173171887</v>
+      </c>
+      <c r="H80" t="n">
         <v>-0.5491332173895884</v>
       </c>
-      <c r="G80" t="n">
+      <c r="I80" t="n">
         <v>1.475341631826585e-07</v>
       </c>
-      <c r="H80" t="n">
+      <c r="J80" t="n">
+        <v>2.273477268716377e-07</v>
+      </c>
+      <c r="K80" t="n">
         <v>18</v>
       </c>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr">
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
+      <c r="P80" t="inlineStr">
         <is>
           <t>CKS1B</t>
         </is>
@@ -3723,24 +4644,36 @@
         <v>0.6074587448528381</v>
       </c>
       <c r="F81" t="n">
+        <v>0.6139905593136213</v>
+      </c>
+      <c r="G81" t="n">
+        <v>-1.012028474786338</v>
+      </c>
+      <c r="H81" t="n">
         <v>-0.558104290185654</v>
       </c>
-      <c r="G81" t="n">
+      <c r="I81" t="n">
         <v>1.936826674020467e-09</v>
       </c>
-      <c r="H81" t="n">
+      <c r="J81" t="n">
+        <v>3.715545048120895e-09</v>
+      </c>
+      <c r="K81" t="n">
         <v>42</v>
       </c>
-      <c r="I81" t="n">
+      <c r="L81" t="n">
         <v>41</v>
       </c>
-      <c r="J81" t="n">
+      <c r="M81" t="n">
         <v>-0.4000278903243101</v>
       </c>
-      <c r="K81" t="n">
+      <c r="N81" t="n">
         <v>0.0008166135159425</v>
       </c>
-      <c r="L81" t="inlineStr">
+      <c r="O81" t="n">
+        <v>0.0009367037388752205</v>
+      </c>
+      <c r="P81" t="inlineStr">
         <is>
           <t>PAICS</t>
         </is>
@@ -3767,18 +4700,28 @@
         <v>3.619375649710779e-05</v>
       </c>
       <c r="F82" t="n">
+        <v>6.075380554871665e-05</v>
+      </c>
+      <c r="G82" t="n">
+        <v>-2.004145108267159</v>
+      </c>
+      <c r="H82" t="n">
         <v>-0.5489886334270651</v>
       </c>
-      <c r="G82" t="n">
+      <c r="I82" t="n">
         <v>2.42813787730849e-05</v>
       </c>
-      <c r="H82" t="n">
+      <c r="J82" t="n">
+        <v>3.136226151334488e-05</v>
+      </c>
+      <c r="K82" t="n">
         <v>18</v>
       </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr">
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr"/>
+      <c r="P82" t="inlineStr">
         <is>
           <t>ELOB</t>
         </is>
@@ -3805,18 +4748,28 @@
         <v>0.0002699866717892</v>
       </c>
       <c r="F83" t="n">
+        <v>0.0003732168698262</v>
+      </c>
+      <c r="G83" t="n">
+        <v>-1.022686670993109</v>
+      </c>
+      <c r="H83" t="n">
         <v>-0.5474675645050944</v>
       </c>
-      <c r="G83" t="n">
+      <c r="I83" t="n">
         <v>2.096596770316438e-07</v>
       </c>
-      <c r="H83" t="n">
+      <c r="J83" t="n">
+        <v>3.128255498567384e-07</v>
+      </c>
+      <c r="K83" t="n">
         <v>59</v>
       </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr">
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr"/>
+      <c r="P83" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -3843,18 +4796,28 @@
         <v>0.0001733636815278</v>
       </c>
       <c r="F84" t="n">
+        <v>0.0002469119100547</v>
+      </c>
+      <c r="G84" t="n">
+        <v>-1.509491831303903</v>
+      </c>
+      <c r="H84" t="n">
         <v>-0.5356546034820067</v>
       </c>
-      <c r="G84" t="n">
+      <c r="I84" t="n">
         <v>0.0003425784512711</v>
       </c>
-      <c r="H84" t="n">
+      <c r="J84" t="n">
+        <v>0.000365936072948675</v>
+      </c>
+      <c r="K84" t="n">
         <v>48</v>
       </c>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr">
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
+      <c r="P84" t="inlineStr">
         <is>
           <t>SCAP</t>
         </is>
@@ -3881,24 +4844,36 @@
         <v>7.29595575325603e-06</v>
       </c>
       <c r="F85" t="n">
+        <v>1.399632328175646e-05</v>
+      </c>
+      <c r="G85" t="n">
+        <v>-1.7196491711041</v>
+      </c>
+      <c r="H85" t="n">
         <v>-0.5371910638437667</v>
       </c>
-      <c r="G85" t="n">
+      <c r="I85" t="n">
         <v>9.001005735746253e-14</v>
       </c>
-      <c r="H85" t="n">
+      <c r="J85" t="n">
+        <v>2.917567376414303e-13</v>
+      </c>
+      <c r="K85" t="n">
         <v>42</v>
       </c>
-      <c r="I85" t="n">
+      <c r="L85" t="n">
         <v>41</v>
       </c>
-      <c r="J85" t="n">
+      <c r="M85" t="n">
         <v>-0.9241258948012384</v>
       </c>
-      <c r="K85" t="n">
+      <c r="N85" t="n">
         <v>2.227747506688165e-10</v>
       </c>
-      <c r="L85" t="inlineStr">
+      <c r="O85" t="n">
+        <v>9.653572528982045e-10</v>
+      </c>
+      <c r="P85" t="inlineStr">
         <is>
           <t>DNM2</t>
         </is>
@@ -3925,18 +4900,28 @@
         <v>7.281066572836062e-05</v>
       </c>
       <c r="F86" t="n">
+        <v>0.0001122000422699</v>
+      </c>
+      <c r="G86" t="n">
+        <v>-1.054139446371316</v>
+      </c>
+      <c r="H86" t="n">
         <v>-0.5296265403183446</v>
       </c>
-      <c r="G86" t="n">
+      <c r="I86" t="n">
         <v>2.748653743555033e-05</v>
       </c>
-      <c r="H86" t="n">
+      <c r="J86" t="n">
+        <v>3.491533133705042e-05</v>
+      </c>
+      <c r="K86" t="n">
         <v>25</v>
       </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr">
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
+      <c r="P86" t="inlineStr">
         <is>
           <t>PTK2</t>
         </is>
@@ -3963,18 +4948,28 @@
         <v>8.942619651372594e-06</v>
       </c>
       <c r="F87" t="n">
+        <v>1.648247543586321e-05</v>
+      </c>
+      <c r="G87" t="n">
+        <v>-1.078034845268306</v>
+      </c>
+      <c r="H87" t="n">
         <v>-0.5274322455253366</v>
       </c>
-      <c r="G87" t="n">
+      <c r="I87" t="n">
         <v>8.274002124418568e-08</v>
       </c>
-      <c r="H87" t="n">
+      <c r="J87" t="n">
+        <v>1.388850356598831e-07</v>
+      </c>
+      <c r="K87" t="n">
         <v>48</v>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr">
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
+      <c r="P87" t="inlineStr">
         <is>
           <t>CFLAR</t>
         </is>
@@ -4001,18 +4996,28 @@
         <v>1.335944354365068e-05</v>
       </c>
       <c r="F88" t="n">
+        <v>2.4149763328907e-05</v>
+      </c>
+      <c r="G88" t="n">
+        <v>-1.131728656938623</v>
+      </c>
+      <c r="H88" t="n">
         <v>-0.5244061909141207</v>
       </c>
-      <c r="G88" t="n">
+      <c r="I88" t="n">
         <v>0.0003911495673497</v>
       </c>
-      <c r="H88" t="n">
+      <c r="J88" t="n">
+        <v>0.0004055298096389583</v>
+      </c>
+      <c r="K88" t="n">
         <v>18</v>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr">
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
+      <c r="P88" t="inlineStr">
         <is>
           <t>CUL2</t>
         </is>
@@ -4039,24 +5044,36 @@
         <v>1.855517055171026e-05</v>
       </c>
       <c r="F89" t="n">
+        <v>3.290917041246727e-05</v>
+      </c>
+      <c r="G89" t="n">
+        <v>-1.019572670762451</v>
+      </c>
+      <c r="H89" t="n">
         <v>-0.5233937049142166</v>
       </c>
-      <c r="G89" t="n">
+      <c r="I89" t="n">
         <v>3.817038605842651e-12</v>
       </c>
-      <c r="H89" t="n">
+      <c r="J89" t="n">
+        <v>1.087277663482452e-11</v>
+      </c>
+      <c r="K89" t="n">
         <v>94</v>
       </c>
-      <c r="I89" t="n">
+      <c r="L89" t="n">
         <v>41</v>
       </c>
-      <c r="J89" t="n">
+      <c r="M89" t="n">
         <v>-0.839487928878518</v>
       </c>
-      <c r="K89" t="n">
+      <c r="N89" t="n">
         <v>4.838733016527725e-08</v>
       </c>
-      <c r="L89" t="inlineStr">
+      <c r="O89" t="n">
+        <v>1.110062280262243e-07</v>
+      </c>
+      <c r="P89" t="inlineStr">
         <is>
           <t>CDK6</t>
         </is>
@@ -4083,24 +5100,36 @@
         <v>4.705664043335697e-08</v>
       </c>
       <c r="F90" t="n">
+        <v>1.228701166870988e-07</v>
+      </c>
+      <c r="G90" t="n">
+        <v>-1.6822690149032</v>
+      </c>
+      <c r="H90" t="n">
         <v>-0.5202424292950369</v>
       </c>
-      <c r="G90" t="n">
+      <c r="I90" t="n">
         <v>1.298972762302589e-23</v>
       </c>
-      <c r="H90" t="n">
+      <c r="J90" t="n">
+        <v>8.140229310429558e-23</v>
+      </c>
+      <c r="K90" t="n">
         <v>94</v>
       </c>
-      <c r="I90" t="n">
+      <c r="L90" t="n">
         <v>41</v>
       </c>
-      <c r="J90" t="n">
+      <c r="M90" t="n">
         <v>-0.891494256708756</v>
       </c>
-      <c r="K90" t="n">
+      <c r="N90" t="n">
         <v>1.133949743113815e-12</v>
       </c>
-      <c r="L90" t="inlineStr">
+      <c r="O90" t="n">
+        <v>1.10560099953597e-11</v>
+      </c>
+      <c r="P90" t="inlineStr">
         <is>
           <t>DNM2</t>
         </is>
@@ -4127,24 +5156,36 @@
         <v>0.0451193928128345</v>
       </c>
       <c r="F91" t="n">
+        <v>0.0481957150500732</v>
+      </c>
+      <c r="G91" t="n">
+        <v>-1.088930411191174</v>
+      </c>
+      <c r="H91" t="n">
         <v>-0.5219999521704304</v>
       </c>
-      <c r="G91" t="n">
+      <c r="I91" t="n">
         <v>1.184437492638099e-07</v>
       </c>
-      <c r="H91" t="n">
+      <c r="J91" t="n">
+        <v>1.919605591516919e-07</v>
+      </c>
+      <c r="K91" t="n">
         <v>42</v>
       </c>
-      <c r="I91" t="n">
+      <c r="L91" t="n">
         <v>41</v>
       </c>
-      <c r="J91" t="n">
+      <c r="M91" t="n">
         <v>-0.646711464571656</v>
       </c>
-      <c r="K91" t="n">
+      <c r="N91" t="n">
         <v>2.704372965473781e-07</v>
       </c>
-      <c r="L91" t="inlineStr">
+      <c r="O91" t="n">
+        <v>5.551081350183024e-07</v>
+      </c>
+      <c r="P91" t="inlineStr">
         <is>
           <t>UROD</t>
         </is>
@@ -4171,18 +5212,28 @@
         <v>3.164132424307008e-14</v>
       </c>
       <c r="F92" t="n">
+        <v>1.416325942308852e-13</v>
+      </c>
+      <c r="G92" t="n">
+        <v>-1.163983595429531</v>
+      </c>
+      <c r="H92" t="n">
         <v>-0.5136822663627335</v>
       </c>
-      <c r="G92" t="n">
+      <c r="I92" t="n">
         <v>5.549757259907932e-10</v>
       </c>
-      <c r="H92" t="n">
+      <c r="J92" t="n">
+        <v>1.159282627625212e-09</v>
+      </c>
+      <c r="K92" t="n">
         <v>63</v>
       </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr">
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr"/>
+      <c r="P92" t="inlineStr">
         <is>
           <t>SCD</t>
         </is>
@@ -4209,18 +5260,28 @@
         <v>9.852205662885487e-07</v>
       </c>
       <c r="F93" t="n">
+        <v>2.058016294024968e-06</v>
+      </c>
+      <c r="G93" t="n">
+        <v>-2.569111507472138</v>
+      </c>
+      <c r="H93" t="n">
         <v>-0.5092316556390317</v>
       </c>
-      <c r="G93" t="n">
+      <c r="I93" t="n">
         <v>1.539485859255806e-06</v>
       </c>
-      <c r="H93" t="n">
+      <c r="J93" t="n">
+        <v>2.159875683135011e-06</v>
+      </c>
+      <c r="K93" t="n">
         <v>48</v>
       </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr">
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
+      <c r="P93" t="inlineStr">
         <is>
           <t>MYC</t>
         </is>
@@ -4247,18 +5308,28 @@
         <v>0.0007320770079146</v>
       </c>
       <c r="F94" t="n">
+        <v>0.0009830748391996</v>
+      </c>
+      <c r="G94" t="n">
+        <v>-1.459898022277849</v>
+      </c>
+      <c r="H94" t="n">
         <v>-0.5090346713123191</v>
       </c>
-      <c r="G94" t="n">
+      <c r="I94" t="n">
         <v>0.0005057623278434</v>
       </c>
-      <c r="H94" t="n">
+      <c r="J94" t="n">
+        <v>0.0005112006324438667</v>
+      </c>
+      <c r="K94" t="n">
         <v>10</v>
       </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr">
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
+      <c r="P94" t="inlineStr">
         <is>
           <t>NCAPD3</t>
         </is>
@@ -4285,18 +5356,28 @@
         <v>3.541373412708916e-06</v>
       </c>
       <c r="F95" t="n">
+        <v>6.935189599888294e-06</v>
+      </c>
+      <c r="G95" t="n">
+        <v>-1.488230514489267</v>
+      </c>
+      <c r="H95" t="n">
         <v>-0.5038775975497989</v>
       </c>
-      <c r="G95" t="n">
+      <c r="I95" t="n">
         <v>2.435579883483166e-05</v>
       </c>
-      <c r="H95" t="n">
+      <c r="J95" t="n">
+        <v>3.136226151334488e-05</v>
+      </c>
+      <c r="K95" t="n">
         <v>53</v>
       </c>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr">
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr"/>
+      <c r="P95" t="inlineStr">
         <is>
           <t>ADSL</t>
         </is>

</xml_diff>

<commit_message>
Blood pairs: growth-pattern adjustment also without the other blood lineage; Sanger replication by lineage group; S3 Table unrounded MDM2 p-values
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S10_Table.xlsx
+++ b/figures/supporting_information/S10_Table.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,13 @@
       <c r="A4" t="inlineStr">
         <is>
           <t>Suspension comparison: lymphoid/myeloid target lineage versus non-blood cell lines annotated as suspension cultures (41 lines); at least ten comparator lines with data required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>*_excl_other_blood: lymphoid/myeloid pairs refitted without the other blood lineage (otherwise the suspension term also absorbs dependencies shared by the two blood lineages); q within the 42 blood pairs.</t>
         </is>
       </c>
     </row>
@@ -468,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P95"/>
+  <dimension ref="A1:T95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -549,6 +556,26 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>coef_unadjusted_excl_other_blood</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>coef_growth_adjusted_excl_other_blood</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>p_growth_adjusted_excl_other_blood</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>q_growth_adjusted_excl_other_blood</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>Gene_symbol</t>
         </is>
       </c>
@@ -595,7 +622,11 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
         <is>
           <t>KRAS</t>
         </is>
@@ -643,7 +674,11 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
         <is>
           <t>SOX10</t>
         </is>
@@ -691,7 +726,11 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
         <is>
           <t>HNF1B</t>
         </is>
@@ -739,7 +778,11 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
         <is>
           <t>FOXA1</t>
         </is>
@@ -787,7 +830,11 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
         <is>
           <t>MDM2</t>
         </is>
@@ -835,7 +882,11 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
         <is>
           <t>CTNNB1</t>
         </is>
@@ -871,7 +922,7 @@
         <v>-1.07582002891723</v>
       </c>
       <c r="I8" t="n">
-        <v>8.069526804470385e-10</v>
+        <v>8.069526804470386e-10</v>
       </c>
       <c r="J8" t="n">
         <v>1.613905360894077e-09</v>
@@ -883,7 +934,11 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
         <is>
           <t>CFLAR</t>
         </is>
@@ -939,7 +994,19 @@
       <c r="O9" t="n">
         <v>7.18998652506705e-13</v>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="P9" t="n">
+        <v>-1.19136688678411</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>-1.090641407667139</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1.511075609412474e-106</v>
+      </c>
+      <c r="S9" t="n">
+        <v>6.346517559532392e-105</v>
+      </c>
+      <c r="T9" t="inlineStr">
         <is>
           <t>MYB</t>
         </is>
@@ -990,12 +1057,24 @@
         <v>-0.9960517864762388</v>
       </c>
       <c r="N10" t="n">
-        <v>6.40991756361763e-13</v>
+        <v>6.409917563617629e-13</v>
       </c>
       <c r="O10" t="n">
-        <v>8.332892832702918e-12</v>
-      </c>
-      <c r="P10" t="inlineStr">
+        <v>8.332892832702916e-12</v>
+      </c>
+      <c r="P10" t="n">
+        <v>-1.108284020148333</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>-1.021266400088498</v>
+      </c>
+      <c r="R10" t="n">
+        <v>2.631529948251494e-36</v>
+      </c>
+      <c r="S10" t="n">
+        <v>2.763106445664068e-35</v>
+      </c>
+      <c r="T10" t="inlineStr">
         <is>
           <t>CBFB</t>
         </is>
@@ -1043,7 +1122,11 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr">
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
         <is>
           <t>TUBB4B</t>
         </is>
@@ -1091,7 +1174,11 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr">
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
         <is>
           <t>PAX8</t>
         </is>
@@ -1139,7 +1226,11 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr">
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
         <is>
           <t>BRAF</t>
         </is>
@@ -1187,7 +1278,11 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr">
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
         <is>
           <t>ZER1</t>
         </is>
@@ -1238,12 +1333,24 @@
         <v>-0.7924728137867726</v>
       </c>
       <c r="N15" t="n">
-        <v>5.203690462565465e-10</v>
+        <v>5.203690462565466e-10</v>
       </c>
       <c r="O15" t="n">
         <v>2.029439280400532e-09</v>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="P15" t="n">
+        <v>-0.8997750419444379</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>-0.6820695286047467</v>
+      </c>
+      <c r="R15" t="n">
+        <v>3.945003076597346e-27</v>
+      </c>
+      <c r="S15" t="n">
+        <v>3.313802584341771e-26</v>
+      </c>
+      <c r="T15" t="inlineStr">
         <is>
           <t>NMNAT1</t>
         </is>
@@ -1299,7 +1406,19 @@
       <c r="O16" t="n">
         <v>8.248875676935083e-09</v>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="P16" t="n">
+        <v>-0.9817466621582834</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>-1.017842197968531</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4.055894175354142e-70</v>
+      </c>
+      <c r="S16" t="n">
+        <v>8.517377768243697e-69</v>
+      </c>
+      <c r="T16" t="inlineStr">
         <is>
           <t>IRF4</t>
         </is>
@@ -1347,7 +1466,11 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
         <is>
           <t>CCND1</t>
         </is>
@@ -1395,7 +1518,11 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -1443,7 +1570,11 @@
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
         <is>
           <t>SKP2</t>
         </is>
@@ -1491,7 +1622,11 @@
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
         <is>
           <t>MDM2</t>
         </is>
@@ -1539,7 +1674,11 @@
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr">
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
         <is>
           <t>MDM2</t>
         </is>
@@ -1587,7 +1726,11 @@
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr">
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
         <is>
           <t>NHLRC2</t>
         </is>
@@ -1635,7 +1778,11 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr">
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
         <is>
           <t>MDM2</t>
         </is>
@@ -1691,7 +1838,19 @@
       <c r="O24" t="n">
         <v>2.286254941101194e-11</v>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="P24" t="n">
+        <v>-0.791464036299235</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>-0.6823994416844057</v>
+      </c>
+      <c r="R24" t="n">
+        <v>6.537333539526764e-44</v>
+      </c>
+      <c r="S24" t="n">
+        <v>9.152266955337469e-43</v>
+      </c>
+      <c r="T24" t="inlineStr">
         <is>
           <t>ATP1B3</t>
         </is>
@@ -1747,7 +1906,19 @@
       <c r="O25" t="n">
         <v>1.163582756351356e-05</v>
       </c>
-      <c r="P25" t="inlineStr">
+      <c r="P25" t="n">
+        <v>-0.6717034994592811</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>-0.5411939530446583</v>
+      </c>
+      <c r="R25" t="n">
+        <v>2.492221828576605e-08</v>
+      </c>
+      <c r="S25" t="n">
+        <v>4.98444365715321e-08</v>
+      </c>
+      <c r="T25" t="inlineStr">
         <is>
           <t>UMPS</t>
         </is>
@@ -1797,7 +1968,19 @@
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr">
+      <c r="P26" t="n">
+        <v>-0.8082968645788399</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>-0.7883820670441467</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0.0141726986520906</v>
+      </c>
+      <c r="S26" t="n">
+        <v>0.0148813335846952</v>
+      </c>
+      <c r="T26" t="inlineStr">
         <is>
           <t>DCAF7</t>
         </is>
@@ -1853,7 +2036,19 @@
       <c r="O27" t="n">
         <v>1.362296852777546e-05</v>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="P27" t="n">
+        <v>-0.6445246980679229</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>-0.3889160583934699</v>
+      </c>
+      <c r="R27" t="n">
+        <v>3.304735589850133e-09</v>
+      </c>
+      <c r="S27" t="n">
+        <v>8.164640869041505e-09</v>
+      </c>
+      <c r="T27" t="inlineStr">
         <is>
           <t>NAMPT</t>
         </is>
@@ -1901,7 +2096,11 @@
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr">
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
         <is>
           <t>SNAP23</t>
         </is>
@@ -1937,10 +2136,10 @@
         <v>-0.7737913303898769</v>
       </c>
       <c r="I29" t="n">
-        <v>4.437835256957793e-29</v>
+        <v>4.437835256957794e-29</v>
       </c>
       <c r="J29" t="n">
-        <v>5.214456426925407e-28</v>
+        <v>5.214456426925408e-28</v>
       </c>
       <c r="K29" t="n">
         <v>94</v>
@@ -1957,7 +2156,19 @@
       <c r="O29" t="n">
         <v>9.30621494027928e-09</v>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="P29" t="n">
+        <v>-0.7356783903575033</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>-0.6444993284928575</v>
+      </c>
+      <c r="R29" t="n">
+        <v>1.287432374846096e-16</v>
+      </c>
+      <c r="S29" t="n">
+        <v>6.008017749281785e-16</v>
+      </c>
+      <c r="T29" t="inlineStr">
         <is>
           <t>UMPS</t>
         </is>
@@ -2005,7 +2216,11 @@
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr">
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
         <is>
           <t>SEPHS2</t>
         </is>
@@ -2061,7 +2276,19 @@
       <c r="O31" t="n">
         <v>9.63481777515442e-05</v>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="P31" t="n">
+        <v>-0.6557923168853583</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>-0.4838541781114725</v>
+      </c>
+      <c r="R31" t="n">
+        <v>1.09263634995528e-06</v>
+      </c>
+      <c r="S31" t="n">
+        <v>1.912113612421741e-06</v>
+      </c>
+      <c r="T31" t="inlineStr">
         <is>
           <t>SEPHS2</t>
         </is>
@@ -2109,7 +2336,11 @@
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr">
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -2165,7 +2396,19 @@
       <c r="O33" t="n">
         <v>7.215472711593775e-06</v>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="P33" t="n">
+        <v>-0.6685931639961885</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>-0.5066744209267507</v>
+      </c>
+      <c r="R33" t="n">
+        <v>1.910261398596061e-08</v>
+      </c>
+      <c r="S33" t="n">
+        <v>4.011548937051728e-08</v>
+      </c>
+      <c r="T33" t="inlineStr">
         <is>
           <t>TFRC</t>
         </is>
@@ -2221,7 +2464,19 @@
       <c r="O34" t="n">
         <v>0.00031401826798901</v>
       </c>
-      <c r="P34" t="inlineStr">
+      <c r="P34" t="n">
+        <v>-0.6574049611373268</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>-0.355825866847508</v>
+      </c>
+      <c r="R34" t="n">
+        <v>1.580824615953873e-05</v>
+      </c>
+      <c r="S34" t="n">
+        <v>2.37123692393081e-05</v>
+      </c>
+      <c r="T34" t="inlineStr">
         <is>
           <t>NAMPT</t>
         </is>
@@ -2277,7 +2532,19 @@
       <c r="O35" t="n">
         <v>3.873572829267974e-09</v>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="P35" t="n">
+        <v>-0.6705232657990701</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>-0.5156538093028626</v>
+      </c>
+      <c r="R35" t="n">
+        <v>4.271533341187661e-13</v>
+      </c>
+      <c r="S35" t="n">
+        <v>1.281460002356298e-12</v>
+      </c>
+      <c r="T35" t="inlineStr">
         <is>
           <t>SDHB</t>
         </is>
@@ -2333,7 +2600,19 @@
       <c r="O36" t="n">
         <v>0.0003363823632088969</v>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="P36" t="n">
+        <v>-0.6826989128180792</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>-0.4493520609110545</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0.0003146152102548</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0.0003990449425068</v>
+      </c>
+      <c r="T36" t="inlineStr">
         <is>
           <t>ADSL</t>
         </is>
@@ -2381,7 +2660,11 @@
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr">
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr">
         <is>
           <t>CCND1</t>
         </is>
@@ -2431,7 +2714,19 @@
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr">
+      <c r="P38" t="n">
+        <v>-0.6195170753125004</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>-0.442817006636708</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0.0186064517830328</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0.01906026768018</v>
+      </c>
+      <c r="T38" t="inlineStr">
         <is>
           <t>SUMO2</t>
         </is>
@@ -2487,7 +2782,19 @@
       <c r="O39" t="n">
         <v>0.003145823582272367</v>
       </c>
-      <c r="P39" t="inlineStr">
+      <c r="P39" t="n">
+        <v>-0.572325575772286</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>-0.2860458867635836</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0.0038694300476111</v>
+      </c>
+      <c r="S39" t="n">
+        <v>0.004392325999991</v>
+      </c>
+      <c r="T39" t="inlineStr">
         <is>
           <t>CDAN1</t>
         </is>
@@ -2543,7 +2850,19 @@
       <c r="O40" t="n">
         <v>3.947540183041832e-10</v>
       </c>
-      <c r="P40" t="inlineStr">
+      <c r="P40" t="n">
+        <v>-0.7314196378528094</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>-0.6680113240951993</v>
+      </c>
+      <c r="R40" t="n">
+        <v>7.793089845435511e-21</v>
+      </c>
+      <c r="S40" t="n">
+        <v>4.675853907261308e-20</v>
+      </c>
+      <c r="T40" t="inlineStr">
         <is>
           <t>EP300</t>
         </is>
@@ -2591,7 +2910,11 @@
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr">
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr">
         <is>
           <t>BCL2L1</t>
         </is>
@@ -2639,7 +2962,11 @@
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr">
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr">
         <is>
           <t>KRAS</t>
         </is>
@@ -2687,7 +3014,11 @@
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr">
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr">
         <is>
           <t>SOX10</t>
         </is>
@@ -2743,7 +3074,19 @@
       <c r="O44" t="n">
         <v>1.889746928966521e-05</v>
       </c>
-      <c r="P44" t="inlineStr">
+      <c r="P44" t="n">
+        <v>-0.699514555562268</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>-0.4550445769623294</v>
+      </c>
+      <c r="R44" t="n">
+        <v>4.107686944514167e-06</v>
+      </c>
+      <c r="S44" t="n">
+        <v>6.635494294984424e-06</v>
+      </c>
+      <c r="T44" t="inlineStr">
         <is>
           <t>ADSL</t>
         </is>
@@ -2791,7 +3134,11 @@
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr">
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr">
         <is>
           <t>SNAP23</t>
         </is>
@@ -2839,7 +3186,11 @@
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr">
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr">
         <is>
           <t>SCAP</t>
         </is>
@@ -2889,7 +3240,19 @@
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr">
+      <c r="P47" t="n">
+        <v>-0.6668828085597043</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>-0.5458106922840568</v>
+      </c>
+      <c r="R47" t="n">
+        <v>0.0021279760657246</v>
+      </c>
+      <c r="S47" t="n">
+        <v>0.0025535712788695</v>
+      </c>
+      <c r="T47" t="inlineStr">
         <is>
           <t>WDR36</t>
         </is>
@@ -2937,7 +3300,11 @@
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr">
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr">
         <is>
           <t>FAM50A</t>
         </is>
@@ -2993,7 +3360,19 @@
       <c r="O49" t="n">
         <v>1.690233774186878e-05</v>
       </c>
-      <c r="P49" t="inlineStr">
+      <c r="P49" t="n">
+        <v>-0.5623571995302931</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>-0.3563639110360637</v>
+      </c>
+      <c r="R49" t="n">
+        <v>8.460773354952871e-09</v>
+      </c>
+      <c r="S49" t="n">
+        <v>1.870276215305371e-08</v>
+      </c>
+      <c r="T49" t="inlineStr">
         <is>
           <t>FPGS</t>
         </is>
@@ -3049,7 +3428,19 @@
       <c r="O50" t="n">
         <v>1.110062280262243e-07</v>
       </c>
-      <c r="P50" t="inlineStr">
+      <c r="P50" t="n">
+        <v>-0.5908623261515948</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>-0.4472366428811658</v>
+      </c>
+      <c r="R50" t="n">
+        <v>1.464077515411452e-13</v>
+      </c>
+      <c r="S50" t="n">
+        <v>4.730096588252382e-13</v>
+      </c>
+      <c r="T50" t="inlineStr">
         <is>
           <t>PAICS</t>
         </is>
@@ -3105,7 +3496,19 @@
       <c r="O51" t="n">
         <v>0.006775903435617779</v>
       </c>
-      <c r="P51" t="inlineStr">
+      <c r="P51" t="n">
+        <v>-0.3995735722582248</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>-0.3863390538494</v>
+      </c>
+      <c r="R51" t="n">
+        <v>0.0089402703325077</v>
+      </c>
+      <c r="S51" t="n">
+        <v>0.0098813514201401</v>
+      </c>
+      <c r="T51" t="inlineStr">
         <is>
           <t>TYMS</t>
         </is>
@@ -3153,7 +3556,11 @@
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr">
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -3209,7 +3616,19 @@
       <c r="O53" t="n">
         <v>0.000517175999192391</v>
       </c>
-      <c r="P53" t="inlineStr">
+      <c r="P53" t="n">
+        <v>-0.3559744783920683</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>-0.350039338621643</v>
+      </c>
+      <c r="R53" t="n">
+        <v>9.429593499497854e-05</v>
+      </c>
+      <c r="S53" t="n">
+        <v>0.0001237634146809</v>
+      </c>
+      <c r="T53" t="inlineStr">
         <is>
           <t>FAM50A</t>
         </is>
@@ -3257,7 +3676,11 @@
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr">
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr">
         <is>
           <t>GRB2</t>
         </is>
@@ -3313,7 +3736,19 @@
       <c r="O55" t="n">
         <v>0.0003363823632088969</v>
       </c>
-      <c r="P55" t="inlineStr">
+      <c r="P55" t="n">
+        <v>-0.4796159686358008</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>-0.4441849152303856</v>
+      </c>
+      <c r="R55" t="n">
+        <v>0.0003230363820293</v>
+      </c>
+      <c r="S55" t="n">
+        <v>0.0003990449425068</v>
+      </c>
+      <c r="T55" t="inlineStr">
         <is>
           <t>DNAJC9</t>
         </is>
@@ -3369,7 +3804,19 @@
       <c r="O56" t="n">
         <v>1.889746928966521e-05</v>
       </c>
-      <c r="P56" t="inlineStr">
+      <c r="P56" t="n">
+        <v>-0.5262970087152592</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>-0.4088222439671773</v>
+      </c>
+      <c r="R56" t="n">
+        <v>2.664139000888552e-05</v>
+      </c>
+      <c r="S56" t="n">
+        <v>3.858408208183421e-05</v>
+      </c>
+      <c r="T56" t="inlineStr">
         <is>
           <t>TRPM7</t>
         </is>
@@ -3417,7 +3864,11 @@
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr">
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr">
         <is>
           <t>CHMP4B</t>
         </is>
@@ -3473,7 +3924,19 @@
       <c r="O58" t="n">
         <v>5.349564181378385e-10</v>
       </c>
-      <c r="P58" t="inlineStr">
+      <c r="P58" t="n">
+        <v>-0.5445253676689159</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>-0.5526040868847748</v>
+      </c>
+      <c r="R58" t="n">
+        <v>1.374573448524384e-13</v>
+      </c>
+      <c r="S58" t="n">
+        <v>4.730096588252382e-13</v>
+      </c>
+      <c r="T58" t="inlineStr">
         <is>
           <t>CTPS1</t>
         </is>
@@ -3529,7 +3992,19 @@
       <c r="O59" t="n">
         <v>7.18998652506705e-13</v>
       </c>
-      <c r="P59" t="inlineStr">
+      <c r="P59" t="n">
+        <v>-0.6126163838317911</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>-0.7478292865875198</v>
+      </c>
+      <c r="R59" t="n">
+        <v>4.584952706748103e-25</v>
+      </c>
+      <c r="S59" t="n">
+        <v>3.209466894723673e-24</v>
+      </c>
+      <c r="T59" t="inlineStr">
         <is>
           <t>CFL1</t>
         </is>
@@ -3577,7 +4052,11 @@
       <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr">
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
+      <c r="T60" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -3633,7 +4112,19 @@
       <c r="O61" t="n">
         <v>0.0002936997942860172</v>
       </c>
-      <c r="P61" t="inlineStr">
+      <c r="P61" t="n">
+        <v>-0.6702735960096563</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>-0.4811393899392877</v>
+      </c>
+      <c r="R61" t="n">
+        <v>3.034127803667951e-05</v>
+      </c>
+      <c r="S61" t="n">
+        <v>4.247778925135131e-05</v>
+      </c>
+      <c r="T61" t="inlineStr">
         <is>
           <t>TFRC</t>
         </is>
@@ -3681,7 +4172,11 @@
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr">
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr">
         <is>
           <t>FAM50A</t>
         </is>
@@ -3737,7 +4232,19 @@
       <c r="O63" t="n">
         <v>0.01741511243142933</v>
       </c>
-      <c r="P63" t="inlineStr">
+      <c r="P63" t="n">
+        <v>-0.499170002701915</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>-0.3093407583952859</v>
+      </c>
+      <c r="R63" t="n">
+        <v>0.0136879440488612</v>
+      </c>
+      <c r="S63" t="n">
+        <v>0.0147408628218505</v>
+      </c>
+      <c r="T63" t="inlineStr">
         <is>
           <t>SEPHS2</t>
         </is>
@@ -3785,7 +4292,11 @@
       <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr">
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr"/>
+      <c r="T64" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -3833,7 +4344,11 @@
       <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr">
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
+      <c r="T65" t="inlineStr">
         <is>
           <t>INTS6</t>
         </is>
@@ -3881,7 +4396,11 @@
       <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr">
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr">
         <is>
           <t>CCND1</t>
         </is>
@@ -3937,7 +4456,19 @@
       <c r="O67" t="n">
         <v>3.947540183041832e-10</v>
       </c>
-      <c r="P67" t="inlineStr">
+      <c r="P67" t="n">
+        <v>-0.463480682827721</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>-0.5663813965520188</v>
+      </c>
+      <c r="R67" t="n">
+        <v>2.408446490320979e-12</v>
+      </c>
+      <c r="S67" t="n">
+        <v>6.743650172898739e-12</v>
+      </c>
+      <c r="T67" t="inlineStr">
         <is>
           <t>UROD</t>
         </is>
@@ -3985,7 +4516,11 @@
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr">
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr">
         <is>
           <t>GRB2</t>
         </is>
@@ -4041,7 +4576,19 @@
       <c r="O69" t="n">
         <v>1.799747931923173e-06</v>
       </c>
-      <c r="P69" t="inlineStr">
+      <c r="P69" t="n">
+        <v>-0.5756765928584637</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>-0.4331177593834895</v>
+      </c>
+      <c r="R69" t="n">
+        <v>8.677271797084175e-07</v>
+      </c>
+      <c r="S69" t="n">
+        <v>1.614892606349051e-06</v>
+      </c>
+      <c r="T69" t="inlineStr">
         <is>
           <t>SDHB</t>
         </is>
@@ -4097,7 +4644,19 @@
       <c r="O70" t="n">
         <v>9.310742874236628e-08</v>
       </c>
-      <c r="P70" t="inlineStr">
+      <c r="P70" t="n">
+        <v>-0.6398112882658535</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>-0.6019968834116127</v>
+      </c>
+      <c r="R70" t="n">
+        <v>1.141964057282769e-11</v>
+      </c>
+      <c r="S70" t="n">
+        <v>2.997655650367268e-11</v>
+      </c>
+      <c r="T70" t="inlineStr">
         <is>
           <t>AP2S1</t>
         </is>
@@ -4145,7 +4704,11 @@
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
-      <c r="P71" t="inlineStr">
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr">
         <is>
           <t>GRB2</t>
         </is>
@@ -4193,7 +4756,11 @@
       <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr"/>
-      <c r="P72" t="inlineStr">
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr">
         <is>
           <t>CHMP4B</t>
         </is>
@@ -4241,7 +4808,11 @@
       <c r="M73" t="inlineStr"/>
       <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr"/>
-      <c r="P73" t="inlineStr">
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr">
         <is>
           <t>CCND1</t>
         </is>
@@ -4297,7 +4868,19 @@
       <c r="O74" t="n">
         <v>5.189250665516321e-08</v>
       </c>
-      <c r="P74" t="inlineStr">
+      <c r="P74" t="n">
+        <v>-0.5401924179280889</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>-0.5418172229337404</v>
+      </c>
+      <c r="R74" t="n">
+        <v>5.261576504866698e-09</v>
+      </c>
+      <c r="S74" t="n">
+        <v>1.227701184468896e-08</v>
+      </c>
+      <c r="T74" t="inlineStr">
         <is>
           <t>CTPS1</t>
         </is>
@@ -4345,7 +4928,11 @@
       <c r="M75" t="inlineStr"/>
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr"/>
-      <c r="P75" t="inlineStr">
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr">
         <is>
           <t>SNAP23</t>
         </is>
@@ -4401,7 +4988,19 @@
       <c r="O76" t="n">
         <v>0.052648770197993</v>
       </c>
-      <c r="P76" t="inlineStr">
+      <c r="P76" t="n">
+        <v>-0.5410462366858577</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>-0.2707626825603527</v>
+      </c>
+      <c r="R76" t="n">
+        <v>0.0322417922244778</v>
+      </c>
+      <c r="S76" t="n">
+        <v>0.0322417922244778</v>
+      </c>
+      <c r="T76" t="inlineStr">
         <is>
           <t>CDAN1</t>
         </is>
@@ -4457,7 +5056,19 @@
       <c r="O77" t="n">
         <v>0.001967497356073191</v>
       </c>
-      <c r="P77" t="inlineStr">
+      <c r="P77" t="n">
+        <v>-0.3468638004781925</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>-0.3282586976917905</v>
+      </c>
+      <c r="R77" t="n">
+        <v>0.0033890974353183</v>
+      </c>
+      <c r="S77" t="n">
+        <v>0.0039539470078713</v>
+      </c>
+      <c r="T77" t="inlineStr">
         <is>
           <t>FAM50A</t>
         </is>
@@ -4513,7 +5124,19 @@
       <c r="O78" t="n">
         <v>1.876700266904672e-07</v>
       </c>
-      <c r="P78" t="inlineStr">
+      <c r="P78" t="n">
+        <v>-0.5076746787411375</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>-0.5289056492437357</v>
+      </c>
+      <c r="R78" t="n">
+        <v>8.843459510959089e-07</v>
+      </c>
+      <c r="S78" t="n">
+        <v>1.614892606349051e-06</v>
+      </c>
+      <c r="T78" t="inlineStr">
         <is>
           <t>MED1</t>
         </is>
@@ -4569,7 +5192,19 @@
       <c r="O79" t="n">
         <v>5.611641928819553e-05</v>
       </c>
-      <c r="P79" t="inlineStr">
+      <c r="P79" t="n">
+        <v>-0.5135429402547746</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>-0.3492822908622425</v>
+      </c>
+      <c r="R79" t="n">
+        <v>8.945287336425944e-06</v>
+      </c>
+      <c r="S79" t="n">
+        <v>1.391489141221813e-05</v>
+      </c>
+      <c r="T79" t="inlineStr">
         <is>
           <t>DHFR</t>
         </is>
@@ -4617,7 +5252,11 @@
       <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr"/>
-      <c r="P80" t="inlineStr">
+      <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr"/>
+      <c r="T80" t="inlineStr">
         <is>
           <t>CKS1B</t>
         </is>
@@ -4673,7 +5312,19 @@
       <c r="O81" t="n">
         <v>0.0009367037388752205</v>
       </c>
-      <c r="P81" t="inlineStr">
+      <c r="P81" t="n">
+        <v>-0.4385907206972599</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>-0.298367592746348</v>
+      </c>
+      <c r="R81" t="n">
+        <v>7.988464419551615e-05</v>
+      </c>
+      <c r="S81" t="n">
+        <v>0.0001082308082648</v>
+      </c>
+      <c r="T81" t="inlineStr">
         <is>
           <t>PAICS</t>
         </is>
@@ -4721,7 +5372,11 @@
       <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr"/>
       <c r="O82" t="inlineStr"/>
-      <c r="P82" t="inlineStr">
+      <c r="P82" t="inlineStr"/>
+      <c r="Q82" t="inlineStr"/>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr"/>
+      <c r="T82" t="inlineStr">
         <is>
           <t>ELOB</t>
         </is>
@@ -4769,7 +5424,11 @@
       <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
-      <c r="P83" t="inlineStr">
+      <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="inlineStr"/>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr"/>
+      <c r="T83" t="inlineStr">
         <is>
           <t>FERMT2</t>
         </is>
@@ -4817,7 +5476,11 @@
       <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr"/>
-      <c r="P84" t="inlineStr">
+      <c r="P84" t="inlineStr"/>
+      <c r="Q84" t="inlineStr"/>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr"/>
+      <c r="T84" t="inlineStr">
         <is>
           <t>SCAP</t>
         </is>
@@ -4873,7 +5536,19 @@
       <c r="O85" t="n">
         <v>9.653572528982045e-10</v>
       </c>
-      <c r="P85" t="inlineStr">
+      <c r="P85" t="n">
+        <v>-0.6877680293398976</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>-0.8422389450349099</v>
+      </c>
+      <c r="R85" t="n">
+        <v>3.647563243378535e-15</v>
+      </c>
+      <c r="S85" t="n">
+        <v>1.531976562218985e-14</v>
+      </c>
+      <c r="T85" t="inlineStr">
         <is>
           <t>DNM2</t>
         </is>
@@ -4921,7 +5596,11 @@
       <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr"/>
       <c r="O86" t="inlineStr"/>
-      <c r="P86" t="inlineStr">
+      <c r="P86" t="inlineStr"/>
+      <c r="Q86" t="inlineStr"/>
+      <c r="R86" t="inlineStr"/>
+      <c r="S86" t="inlineStr"/>
+      <c r="T86" t="inlineStr">
         <is>
           <t>PTK2</t>
         </is>
@@ -4969,7 +5648,11 @@
       <c r="M87" t="inlineStr"/>
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr"/>
-      <c r="P87" t="inlineStr">
+      <c r="P87" t="inlineStr"/>
+      <c r="Q87" t="inlineStr"/>
+      <c r="R87" t="inlineStr"/>
+      <c r="S87" t="inlineStr"/>
+      <c r="T87" t="inlineStr">
         <is>
           <t>CFLAR</t>
         </is>
@@ -5017,7 +5700,11 @@
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
-      <c r="P88" t="inlineStr">
+      <c r="P88" t="inlineStr"/>
+      <c r="Q88" t="inlineStr"/>
+      <c r="R88" t="inlineStr"/>
+      <c r="S88" t="inlineStr"/>
+      <c r="T88" t="inlineStr">
         <is>
           <t>CUL2</t>
         </is>
@@ -5073,7 +5760,19 @@
       <c r="O89" t="n">
         <v>1.110062280262243e-07</v>
       </c>
-      <c r="P89" t="inlineStr">
+      <c r="P89" t="n">
+        <v>-0.5126079853638232</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>-0.6448054359569048</v>
+      </c>
+      <c r="R89" t="n">
+        <v>8.596751161173015e-14</v>
+      </c>
+      <c r="S89" t="n">
+        <v>3.282395897902423e-13</v>
+      </c>
+      <c r="T89" t="inlineStr">
         <is>
           <t>CDK6</t>
         </is>
@@ -5100,7 +5799,7 @@
         <v>4.705664043335697e-08</v>
       </c>
       <c r="F90" t="n">
-        <v>1.228701166870988e-07</v>
+        <v>1.228701166870987e-07</v>
       </c>
       <c r="G90" t="n">
         <v>-1.6822690149032</v>
@@ -5129,7 +5828,19 @@
       <c r="O90" t="n">
         <v>1.10560099953597e-11</v>
       </c>
-      <c r="P90" t="inlineStr">
+      <c r="P90" t="n">
+        <v>-0.5774524764600292</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>-0.763783179065633</v>
+      </c>
+      <c r="R90" t="n">
+        <v>1.691064228158077e-19</v>
+      </c>
+      <c r="S90" t="n">
+        <v>8.878087197829902e-19</v>
+      </c>
+      <c r="T90" t="inlineStr">
         <is>
           <t>DNM2</t>
         </is>
@@ -5185,7 +5896,19 @@
       <c r="O91" t="n">
         <v>5.551081350183024e-07</v>
       </c>
-      <c r="P91" t="inlineStr">
+      <c r="P91" t="n">
+        <v>-0.4161962126920852</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>-0.4852044571786227</v>
+      </c>
+      <c r="R91" t="n">
+        <v>1.888785179370901e-06</v>
+      </c>
+      <c r="S91" t="n">
+        <v>3.173159101343113e-06</v>
+      </c>
+      <c r="T91" t="inlineStr">
         <is>
           <t>UROD</t>
         </is>
@@ -5233,7 +5956,11 @@
       <c r="M92" t="inlineStr"/>
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr"/>
-      <c r="P92" t="inlineStr">
+      <c r="P92" t="inlineStr"/>
+      <c r="Q92" t="inlineStr"/>
+      <c r="R92" t="inlineStr"/>
+      <c r="S92" t="inlineStr"/>
+      <c r="T92" t="inlineStr">
         <is>
           <t>SCD</t>
         </is>
@@ -5281,7 +6008,11 @@
       <c r="M93" t="inlineStr"/>
       <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr"/>
-      <c r="P93" t="inlineStr">
+      <c r="P93" t="inlineStr"/>
+      <c r="Q93" t="inlineStr"/>
+      <c r="R93" t="inlineStr"/>
+      <c r="S93" t="inlineStr"/>
+      <c r="T93" t="inlineStr">
         <is>
           <t>MYC</t>
         </is>
@@ -5329,7 +6060,11 @@
       <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr"/>
       <c r="O94" t="inlineStr"/>
-      <c r="P94" t="inlineStr">
+      <c r="P94" t="inlineStr"/>
+      <c r="Q94" t="inlineStr"/>
+      <c r="R94" t="inlineStr"/>
+      <c r="S94" t="inlineStr"/>
+      <c r="T94" t="inlineStr">
         <is>
           <t>NCAPD3</t>
         </is>
@@ -5377,7 +6112,11 @@
       <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
-      <c r="P95" t="inlineStr">
+      <c r="P95" t="inlineStr"/>
+      <c r="Q95" t="inlineStr"/>
+      <c r="R95" t="inlineStr"/>
+      <c r="S95" t="inlineStr"/>
+      <c r="T95" t="inlineStr">
         <is>
           <t>ADSL</t>
         </is>

</xml_diff>

<commit_message>
All OLS inference with HC3 heteroscedasticity-robust standard errors (t reference): part2, growth_confound, revision4, revision6; robust_se_checks.py
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S10_Table.xlsx
+++ b/figures/supporting_information/S10_Table.xlsx
@@ -598,10 +598,10 @@
         <v>-1.466629990742004</v>
       </c>
       <c r="E2" t="n">
-        <v>1.643433183919731e-59</v>
+        <v>9.2381806992057e-24</v>
       </c>
       <c r="F2" t="n">
-        <v>2.574711988140911e-58</v>
+        <v>4.341944928626679e-22</v>
       </c>
       <c r="G2" t="n">
         <v>-2.086661855015164</v>
@@ -650,10 +650,10 @@
         <v>-1.218145757229453</v>
       </c>
       <c r="E3" t="n">
-        <v>3.442602794463395e-152</v>
+        <v>4.193172326733162e-34</v>
       </c>
       <c r="F3" t="n">
-        <v>3.236046626795591e-150</v>
+        <v>3.941581987129173e-32</v>
       </c>
       <c r="G3" t="n">
         <v>-1.670194030844392</v>
@@ -702,10 +702,10 @@
         <v>-1.037557449728486</v>
       </c>
       <c r="E4" t="n">
-        <v>1.122464150335925e-40</v>
+        <v>3.716581000536629e-10</v>
       </c>
       <c r="F4" t="n">
-        <v>1.17235144590641e-39</v>
+        <v>1.746793070252216e-09</v>
       </c>
       <c r="G4" t="n">
         <v>-1.425133103283988</v>
@@ -754,10 +754,10 @@
         <v>-1.140124286230249</v>
       </c>
       <c r="E5" t="n">
-        <v>1.056809636006767e-15</v>
+        <v>0.0109510455968606</v>
       </c>
       <c r="F5" t="n">
-        <v>6.208756611539757e-15</v>
+        <v>0.0133688089104532</v>
       </c>
       <c r="G5" t="n">
         <v>-1.363840520951394</v>
@@ -806,10 +806,10 @@
         <v>-0.9167465205972932</v>
       </c>
       <c r="E6" t="n">
-        <v>1.913639539971504e-07</v>
+        <v>9.791867439540263e-10</v>
       </c>
       <c r="F6" t="n">
-        <v>4.612361968136446e-07</v>
+        <v>4.183797905985385e-09</v>
       </c>
       <c r="G6" t="n">
         <v>-1.55427191249818</v>
@@ -858,10 +858,10 @@
         <v>-0.9734375633292824</v>
       </c>
       <c r="E7" t="n">
-        <v>4.986058889767983e-92</v>
+        <v>2.026148259516428e-22</v>
       </c>
       <c r="F7" t="n">
-        <v>9.373790712763807e-91</v>
+        <v>4.761448409863607e-21</v>
       </c>
       <c r="G7" t="n">
         <v>-1.255339207492288</v>
@@ -910,10 +910,10 @@
         <v>-0.8751707583059087</v>
       </c>
       <c r="E8" t="n">
-        <v>2.994953655844778e-15</v>
+        <v>1.239849669181991e-09</v>
       </c>
       <c r="F8" t="n">
-        <v>1.564031353607828e-14</v>
+        <v>4.8560778709628e-09</v>
       </c>
       <c r="G8" t="n">
         <v>-1.630766279564239</v>
@@ -962,10 +962,10 @@
         <v>-0.7690624939602465</v>
       </c>
       <c r="E9" t="n">
-        <v>2.597573811120073e-46</v>
+        <v>3.157543237811489e-13</v>
       </c>
       <c r="F9" t="n">
-        <v>3.052149228066087e-45</v>
+        <v>2.698264221402545e-12</v>
       </c>
       <c r="G9" t="n">
         <v>-1.360154978943165</v>
@@ -1001,10 +1001,10 @@
         <v>-1.090641407667139</v>
       </c>
       <c r="R9" t="n">
-        <v>1.511075609412474e-106</v>
+        <v>3.548818659009323e-24</v>
       </c>
       <c r="S9" t="n">
-        <v>6.346517559532392e-105</v>
+        <v>4.968346122613052e-23</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
@@ -1030,10 +1030,10 @@
         <v>-0.5809133381194328</v>
       </c>
       <c r="E10" t="n">
-        <v>5.211680712421602e-15</v>
+        <v>2.327677017404333e-08</v>
       </c>
       <c r="F10" t="n">
-        <v>2.449489934838153e-14</v>
+        <v>7.814344272714545e-08</v>
       </c>
       <c r="G10" t="n">
         <v>-1.23964073579391</v>
@@ -1069,10 +1069,10 @@
         <v>-1.021266400088498</v>
       </c>
       <c r="R10" t="n">
-        <v>2.631529948251494e-36</v>
+        <v>1.669987048266087e-21</v>
       </c>
       <c r="S10" t="n">
-        <v>2.763106445664068e-35</v>
+        <v>1.753486400679392e-20</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -1098,10 +1098,10 @@
         <v>-0.867531635654875</v>
       </c>
       <c r="E11" t="n">
-        <v>1.397146005251066e-07</v>
+        <v>0.0212556734239514</v>
       </c>
       <c r="F11" t="n">
-        <v>3.45609801298948e-07</v>
+        <v>0.0246670778006349</v>
       </c>
       <c r="G11" t="n">
         <v>-1.371058348815747</v>
@@ -1150,10 +1150,10 @@
         <v>-0.8316805340339947</v>
       </c>
       <c r="E12" t="n">
-        <v>1.306927087769899e-47</v>
+        <v>1.80328904062028e-12</v>
       </c>
       <c r="F12" t="n">
-        <v>1.755016375005293e-46</v>
+        <v>1.210779784416474e-11</v>
       </c>
       <c r="G12" t="n">
         <v>-1.119002902546843</v>
@@ -1202,10 +1202,10 @@
         <v>-0.8507937916870913</v>
       </c>
       <c r="E13" t="n">
-        <v>1.17976165263478e-103</v>
+        <v>1.207348665672825e-22</v>
       </c>
       <c r="F13" t="n">
-        <v>5.544879767383465e-102</v>
+        <v>3.783025819108186e-21</v>
       </c>
       <c r="G13" t="n">
         <v>-1.124780833992745</v>
@@ -1254,10 +1254,10 @@
         <v>-0.9279945886442608</v>
       </c>
       <c r="E14" t="n">
-        <v>2.846253139062331e-100</v>
+        <v>1.300849566620287e-12</v>
       </c>
       <c r="F14" t="n">
-        <v>8.918259835728637e-99</v>
+        <v>9.406143020177458e-12</v>
       </c>
       <c r="G14" t="n">
         <v>-1.101619065138771</v>
@@ -1306,10 +1306,10 @@
         <v>-0.6240089631113014</v>
       </c>
       <c r="E15" t="n">
-        <v>5.199182551965316e-30</v>
+        <v>5.297454257283649e-17</v>
       </c>
       <c r="F15" t="n">
-        <v>4.887231598847397e-29</v>
+        <v>7.113724288352328e-16</v>
       </c>
       <c r="G15" t="n">
         <v>-1.200224825187052</v>
@@ -1345,10 +1345,10 @@
         <v>-0.6820695286047467</v>
       </c>
       <c r="R15" t="n">
-        <v>3.945003076597346e-27</v>
+        <v>1.763474593676257e-14</v>
       </c>
       <c r="S15" t="n">
-        <v>3.313802584341771e-26</v>
+        <v>6.733266630400257e-14</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
@@ -1374,10 +1374,10 @@
         <v>-1.014904235790922</v>
       </c>
       <c r="E16" t="n">
-        <v>1.871900046127947e-92</v>
+        <v>1.324149640629335e-20</v>
       </c>
       <c r="F16" t="n">
-        <v>4.398965108400675e-91</v>
+        <v>2.489401324383149e-19</v>
       </c>
       <c r="G16" t="n">
         <v>-1.041153941289623</v>
@@ -1413,10 +1413,10 @@
         <v>-1.017842197968531</v>
       </c>
       <c r="R16" t="n">
-        <v>4.055894175354142e-70</v>
+        <v>1.943051403486079e-16</v>
       </c>
       <c r="S16" t="n">
-        <v>8.517377768243697e-69</v>
+        <v>1.020101986830192e-15</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
@@ -1442,10 +1442,10 @@
         <v>-0.5722740621737636</v>
       </c>
       <c r="E17" t="n">
-        <v>8.823360352502614e-06</v>
+        <v>1.409475115563508e-06</v>
       </c>
       <c r="F17" t="n">
-        <v>1.648247543586321e-05</v>
+        <v>3.397196432383839e-06</v>
       </c>
       <c r="G17" t="n">
         <v>-1.978953338506378</v>
@@ -1494,10 +1494,10 @@
         <v>-0.5765863692280629</v>
       </c>
       <c r="E18" t="n">
-        <v>1.475890482115414e-09</v>
+        <v>2.659301277856699e-07</v>
       </c>
       <c r="F18" t="n">
-        <v>4.954775189958891e-09</v>
+        <v>7.142123431957991e-07</v>
       </c>
       <c r="G18" t="n">
         <v>-1.402905363847756</v>
@@ -1546,10 +1546,10 @@
         <v>-0.816443456107911</v>
       </c>
       <c r="E19" t="n">
-        <v>7.313612224191613e-14</v>
+        <v>3.062138561084342e-05</v>
       </c>
       <c r="F19" t="n">
-        <v>3.124907041245508e-13</v>
+        <v>5.535404321960156e-05</v>
       </c>
       <c r="G19" t="n">
         <v>-1.569685120222577</v>
@@ -1598,10 +1598,10 @@
         <v>-0.6509600366428719</v>
       </c>
       <c r="E20" t="n">
-        <v>1.343649811283425e-11</v>
+        <v>1.498902695124236e-07</v>
       </c>
       <c r="F20" t="n">
-        <v>5.052123290425679e-11</v>
+        <v>4.144025098284654e-07</v>
       </c>
       <c r="G20" t="n">
         <v>-1.285985398539891</v>
@@ -1650,10 +1650,10 @@
         <v>-0.5224082770380014</v>
       </c>
       <c r="E21" t="n">
-        <v>1.99916691160039e-05</v>
+        <v>0.0003730130805074</v>
       </c>
       <c r="F21" t="n">
-        <v>3.480031290563641e-05</v>
+        <v>0.0005748070420933</v>
       </c>
       <c r="G21" t="n">
         <v>-1.278358846210356</v>
@@ -1702,10 +1702,10 @@
         <v>-0.5879818486193304</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0004429851570295</v>
+        <v>0.0018487022660647</v>
       </c>
       <c r="F22" t="n">
-        <v>0.0006034870255184</v>
+        <v>0.0024475776480293</v>
       </c>
       <c r="G22" t="n">
         <v>-1.612606018434213</v>
@@ -1754,10 +1754,10 @@
         <v>-0.5509080354421592</v>
       </c>
       <c r="E23" t="n">
-        <v>6.625351181132343e-17</v>
+        <v>1.238225150972693e-09</v>
       </c>
       <c r="F23" t="n">
-        <v>4.448450078760288e-16</v>
+        <v>4.8560778709628e-09</v>
       </c>
       <c r="G23" t="n">
         <v>-1.200210115640962</v>
@@ -1806,10 +1806,10 @@
         <v>-0.491256413168795</v>
       </c>
       <c r="E24" t="n">
-        <v>1.441800374548279e-28</v>
+        <v>1.07038128890379e-12</v>
       </c>
       <c r="F24" t="n">
-        <v>1.232083956432165e-27</v>
+        <v>8.384653429746356e-12</v>
       </c>
       <c r="G24" t="n">
         <v>-1.110319560589528</v>
@@ -1845,10 +1845,10 @@
         <v>-0.6823994416844057</v>
       </c>
       <c r="R24" t="n">
-        <v>6.537333539526764e-44</v>
+        <v>3.618700172953395e-25</v>
       </c>
       <c r="S24" t="n">
-        <v>9.152266955337469e-43</v>
+        <v>7.59927036320213e-24</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
@@ -1874,10 +1874,10 @@
         <v>-0.1946623767093909</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0212950430011134</v>
+        <v>0.0612258829042377</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0238301671679126</v>
+        <v>0.0646655392471724</v>
       </c>
       <c r="G25" t="n">
         <v>-1.257657148122667</v>
@@ -1913,10 +1913,10 @@
         <v>-0.5411939530446583</v>
       </c>
       <c r="R25" t="n">
-        <v>2.492221828576605e-08</v>
+        <v>4.507360214180825e-06</v>
       </c>
       <c r="S25" t="n">
-        <v>4.98444365715321e-08</v>
+        <v>7.281120345984409e-06</v>
       </c>
       <c r="T25" t="inlineStr">
         <is>
@@ -1942,10 +1942,10 @@
         <v>-0.4892201023435651</v>
       </c>
       <c r="E26" t="n">
-        <v>0.0353499600566551</v>
+        <v>0.0497102394691889</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0381942097163859</v>
+        <v>0.0530995739784517</v>
       </c>
       <c r="G26" t="n">
         <v>-1.437407598292096</v>
@@ -1975,10 +1975,10 @@
         <v>-0.7883820670441467</v>
       </c>
       <c r="R26" t="n">
-        <v>0.0141726986520906</v>
+        <v>3.401060992608954e-06</v>
       </c>
       <c r="S26" t="n">
-        <v>0.0148813335846952</v>
+        <v>5.95185673706567e-06</v>
       </c>
       <c r="T26" t="inlineStr">
         <is>
@@ -2004,10 +2004,10 @@
         <v>-0.2217818300329433</v>
       </c>
       <c r="E27" t="n">
-        <v>9.745357731664092e-05</v>
+        <v>0.0005440571971289</v>
       </c>
       <c r="F27" t="n">
-        <v>0.0001477521978671</v>
+        <v>0.0008117678814304</v>
       </c>
       <c r="G27" t="n">
         <v>-1.082122273813447</v>
@@ -2043,10 +2043,10 @@
         <v>-0.3889160583934699</v>
       </c>
       <c r="R27" t="n">
-        <v>3.304735589850133e-09</v>
+        <v>3.429715997380514e-07</v>
       </c>
       <c r="S27" t="n">
-        <v>8.164640869041505e-09</v>
+        <v>6.262959647390503e-07</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
@@ -2072,10 +2072,10 @@
         <v>-0.6331997337656251</v>
       </c>
       <c r="E28" t="n">
-        <v>1.630459465092921e-13</v>
+        <v>2.486823118581729e-10</v>
       </c>
       <c r="F28" t="n">
-        <v>6.663616944292809e-13</v>
+        <v>1.298674295259347e-09</v>
       </c>
       <c r="G28" t="n">
         <v>-1.522591615377213</v>
@@ -2124,10 +2124,10 @@
         <v>-0.3945028520116778</v>
       </c>
       <c r="E29" t="n">
-        <v>7.572587350113489e-09</v>
+        <v>2.357711451548007e-06</v>
       </c>
       <c r="F29" t="n">
-        <v>2.296203906163445e-08</v>
+        <v>5.276782772512207e-06</v>
       </c>
       <c r="G29" t="n">
         <v>-1.196063514301491</v>
@@ -2163,10 +2163,10 @@
         <v>-0.6444993284928575</v>
       </c>
       <c r="R29" t="n">
-        <v>1.287432374846096e-16</v>
+        <v>1.712693490700832e-14</v>
       </c>
       <c r="S29" t="n">
-        <v>6.008017749281785e-16</v>
+        <v>6.733266630400257e-14</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
@@ -2192,10 +2192,10 @@
         <v>-0.5348262710622504</v>
       </c>
       <c r="E30" t="n">
-        <v>4.510072204204106e-07</v>
+        <v>5.1176326787884e-05</v>
       </c>
       <c r="F30" t="n">
-        <v>1.0340165541346e-06</v>
+        <v>8.590311996537671e-05</v>
       </c>
       <c r="G30" t="n">
         <v>-1.461931445337405</v>
@@ -2244,10 +2244,10 @@
         <v>-0.345797966152031</v>
       </c>
       <c r="E31" t="n">
-        <v>5.00326172621582e-05</v>
+        <v>8.112077236396088e-06</v>
       </c>
       <c r="F31" t="n">
-        <v>8.108734521798054e-05</v>
+        <v>1.657685348307027e-05</v>
       </c>
       <c r="G31" t="n">
         <v>-1.414330407664655</v>
@@ -2283,10 +2283,10 @@
         <v>-0.4838541781114725</v>
       </c>
       <c r="R31" t="n">
-        <v>1.09263634995528e-06</v>
+        <v>1.484367158099037e-07</v>
       </c>
       <c r="S31" t="n">
-        <v>1.912113612421741e-06</v>
+        <v>2.833791847279979e-07</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
@@ -2312,10 +2312,10 @@
         <v>-0.5156905391930441</v>
       </c>
       <c r="E32" t="n">
-        <v>2.893712982107823e-15</v>
+        <v>1.905506261249614e-11</v>
       </c>
       <c r="F32" t="n">
-        <v>1.564031353607828e-14</v>
+        <v>1.119484928484148e-10</v>
       </c>
       <c r="G32" t="n">
         <v>-1.234013429452743</v>
@@ -2364,10 +2364,10 @@
         <v>-0.2965941221965927</v>
       </c>
       <c r="E33" t="n">
-        <v>0.0001339470885691</v>
+        <v>1.550723167285811e-05</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0001967347863358</v>
+        <v>3.036832869268046e-05</v>
       </c>
       <c r="G33" t="n">
         <v>-1.575504219990485</v>
@@ -2403,10 +2403,10 @@
         <v>-0.5066744209267507</v>
       </c>
       <c r="R33" t="n">
-        <v>1.910261398596061e-08</v>
+        <v>7.907978583453246e-10</v>
       </c>
       <c r="S33" t="n">
-        <v>4.011548937051728e-08</v>
+        <v>2.075844378156477e-09</v>
       </c>
       <c r="T33" t="inlineStr">
         <is>
@@ -2432,10 +2432,10 @@
         <v>-0.1731880034354361</v>
       </c>
       <c r="E34" t="n">
-        <v>0.0135991678847403</v>
+        <v>0.0230961179890758</v>
       </c>
       <c r="F34" t="n">
-        <v>0.0157817503847603</v>
+        <v>0.0261570492888328</v>
       </c>
       <c r="G34" t="n">
         <v>-1.056576298494927</v>
@@ -2471,10 +2471,10 @@
         <v>-0.355825866847508</v>
       </c>
       <c r="R34" t="n">
-        <v>1.580824615953873e-05</v>
+        <v>0.0005841573048545</v>
       </c>
       <c r="S34" t="n">
-        <v>2.37123692393081e-05</v>
+        <v>0.0006815168556636</v>
       </c>
       <c r="T34" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         <v>-0.3394202337783599</v>
       </c>
       <c r="E35" t="n">
-        <v>2.759659594195708e-08</v>
+        <v>4.058675133120099e-08</v>
       </c>
       <c r="F35" t="n">
-        <v>7.629647113364603e-08</v>
+        <v>1.315570560390653e-07</v>
       </c>
       <c r="G35" t="n">
         <v>-1.128976862422515</v>
@@ -2539,10 +2539,10 @@
         <v>-0.5156538093028626</v>
       </c>
       <c r="R35" t="n">
-        <v>4.271533341187661e-13</v>
+        <v>5.637146619926345e-14</v>
       </c>
       <c r="S35" t="n">
-        <v>1.281460002356298e-12</v>
+        <v>1.973001316974221e-13</v>
       </c>
       <c r="T35" t="inlineStr">
         <is>
@@ -2568,10 +2568,10 @@
         <v>-0.1774614378957123</v>
       </c>
       <c r="E36" t="n">
-        <v>0.0888406419230869</v>
+        <v>0.0434893210771546</v>
       </c>
       <c r="F36" t="n">
-        <v>0.09383168922213669</v>
+        <v>0.0469884618534773</v>
       </c>
       <c r="G36" t="n">
         <v>-1.699645549757265</v>
@@ -2607,10 +2607,10 @@
         <v>-0.4493520609110545</v>
       </c>
       <c r="R36" t="n">
-        <v>0.0003146152102548</v>
+        <v>0.000157835874102</v>
       </c>
       <c r="S36" t="n">
-        <v>0.0003990449425068</v>
+        <v>0.0002071595847588</v>
       </c>
       <c r="T36" t="inlineStr">
         <is>
@@ -2636,10 +2636,10 @@
         <v>-0.4250005033463671</v>
       </c>
       <c r="E37" t="n">
-        <v>3.83348282584508e-05</v>
+        <v>8.081446708089195e-05</v>
       </c>
       <c r="F37" t="n">
-        <v>6.321883958411185e-05</v>
+        <v>0.0001332729808</v>
       </c>
       <c r="G37" t="n">
         <v>-1.796984303523731</v>
@@ -2688,10 +2688,10 @@
         <v>-0.4415626374051086</v>
       </c>
       <c r="E38" t="n">
-        <v>0.0148884280757132</v>
+        <v>0.0358207889804875</v>
       </c>
       <c r="F38" t="n">
-        <v>0.0170672224282565</v>
+        <v>0.039152955397277</v>
       </c>
       <c r="G38" t="n">
         <v>-1.514616136205607</v>
@@ -2721,10 +2721,10 @@
         <v>-0.442817006636708</v>
       </c>
       <c r="R38" t="n">
-        <v>0.0186064517830328</v>
+        <v>0.0360911143676149</v>
       </c>
       <c r="S38" t="n">
-        <v>0.01906026768018</v>
+        <v>0.0360911143676149</v>
       </c>
       <c r="T38" t="inlineStr">
         <is>
@@ -2750,10 +2750,10 @@
         <v>-0.1864190442937805</v>
       </c>
       <c r="E39" t="n">
-        <v>0.0292194528351796</v>
+        <v>0.0216512579329149</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0323132772530221</v>
+        <v>0.0248197347035853</v>
       </c>
       <c r="G39" t="n">
         <v>-1.63442958182128</v>
@@ -2789,10 +2789,10 @@
         <v>-0.2860458867635836</v>
       </c>
       <c r="R39" t="n">
-        <v>0.0038694300476111</v>
+        <v>0.0022542614641677</v>
       </c>
       <c r="S39" t="n">
-        <v>0.004392325999991</v>
+        <v>0.002558891391758</v>
       </c>
       <c r="T39" t="inlineStr">
         <is>
@@ -2818,10 +2818,10 @@
         <v>-0.5565213244128032</v>
       </c>
       <c r="E40" t="n">
-        <v>2.090280984449076e-19</v>
+        <v>2.620912160502158e-15</v>
       </c>
       <c r="F40" t="n">
-        <v>1.637386771151776e-18</v>
+        <v>2.737397145413365e-14</v>
       </c>
       <c r="G40" t="n">
         <v>-1.004941145021997</v>
@@ -2857,10 +2857,10 @@
         <v>-0.6680113240951993</v>
       </c>
       <c r="R40" t="n">
-        <v>7.793089845435511e-21</v>
+        <v>1.782767193299237e-19</v>
       </c>
       <c r="S40" t="n">
-        <v>4.675853907261308e-20</v>
+        <v>1.497524442371358e-18</v>
       </c>
       <c r="T40" t="inlineStr">
         <is>
@@ -2886,10 +2886,10 @@
         <v>-0.5926561902242218</v>
       </c>
       <c r="E41" t="n">
-        <v>3.592411582983894e-11</v>
+        <v>1.089871834729226e-08</v>
       </c>
       <c r="F41" t="n">
-        <v>1.298794956924946e-10</v>
+        <v>3.940305864021046e-08</v>
       </c>
       <c r="G41" t="n">
         <v>-1.673854449943091</v>
@@ -2938,10 +2938,10 @@
         <v>-0.7317156298179192</v>
       </c>
       <c r="E42" t="n">
-        <v>7.312073568677205e-19</v>
+        <v>3.493687402541418e-10</v>
       </c>
       <c r="F42" t="n">
-        <v>5.28719165735121e-18</v>
+        <v>1.72845587283628e-09</v>
       </c>
       <c r="G42" t="n">
         <v>-1.211311977116099</v>
@@ -2990,10 +2990,10 @@
         <v>-0.7927243145712737</v>
       </c>
       <c r="E43" t="n">
-        <v>1.461590086948102e-08</v>
+        <v>0.004739378576263</v>
       </c>
       <c r="F43" t="n">
-        <v>4.163317217367322e-08</v>
+        <v>0.0059400211489162</v>
       </c>
       <c r="G43" t="n">
         <v>-1.011961766589184</v>
@@ -3042,10 +3042,10 @@
         <v>-0.280350832491644</v>
       </c>
       <c r="E44" t="n">
-        <v>0.0009193810892928</v>
+        <v>0.0003088941421225</v>
       </c>
       <c r="F44" t="n">
-        <v>0.0012172087661059</v>
+        <v>0.0004839341559919</v>
       </c>
       <c r="G44" t="n">
         <v>-1.624021565456589</v>
@@ -3081,10 +3081,10 @@
         <v>-0.4550445769623294</v>
       </c>
       <c r="R44" t="n">
-        <v>4.107686944514167e-06</v>
+        <v>3.613065557839128e-06</v>
       </c>
       <c r="S44" t="n">
-        <v>6.635494294984424e-06</v>
+        <v>6.069950137169735e-06</v>
       </c>
       <c r="T44" t="inlineStr">
         <is>
@@ -3110,10 +3110,10 @@
         <v>-0.5571030444460986</v>
       </c>
       <c r="E45" t="n">
-        <v>0.0001449830829607</v>
+        <v>4.663914935806954e-05</v>
       </c>
       <c r="F45" t="n">
-        <v>0.0002096678430508</v>
+        <v>7.971054617560977e-05</v>
       </c>
       <c r="G45" t="n">
         <v>-1.446877134048081</v>
@@ -3162,10 +3162,10 @@
         <v>-0.5530058691968847</v>
       </c>
       <c r="E46" t="n">
-        <v>3.727226775396882e-08</v>
+        <v>6.591109340452662e-08</v>
       </c>
       <c r="F46" t="n">
-        <v>1.00102661967802e-07</v>
+        <v>1.998594445169517e-07</v>
       </c>
       <c r="G46" t="n">
         <v>-1.656857628342071</v>
@@ -3214,10 +3214,10 @@
         <v>-0.4564794856797313</v>
       </c>
       <c r="E47" t="n">
-        <v>0.002750289889322</v>
+        <v>0.0001577803215791</v>
       </c>
       <c r="F47" t="n">
-        <v>0.0034936114810306</v>
+        <v>0.0002513788174311</v>
       </c>
       <c r="G47" t="n">
         <v>-2.431461893651065</v>
@@ -3247,10 +3247,10 @@
         <v>-0.5458106922840568</v>
       </c>
       <c r="R47" t="n">
-        <v>0.0021279760657246</v>
+        <v>0.0003826743663625</v>
       </c>
       <c r="S47" t="n">
-        <v>0.0025535712788695</v>
+        <v>0.0004592092396351</v>
       </c>
       <c r="T47" t="inlineStr">
         <is>
@@ -3276,10 +3276,10 @@
         <v>-0.3520311337829496</v>
       </c>
       <c r="E48" t="n">
-        <v>8.535856631369382e-07</v>
+        <v>2.517732168808004e-05</v>
       </c>
       <c r="F48" t="n">
-        <v>1.865977961276098e-06</v>
+        <v>4.640525958195145e-05</v>
       </c>
       <c r="G48" t="n">
         <v>-1.137284631353363</v>
@@ -3328,10 +3328,10 @@
         <v>-0.2733534170765126</v>
       </c>
       <c r="E49" t="n">
-        <v>2.74261262861531e-07</v>
+        <v>2.145444120474107e-05</v>
       </c>
       <c r="F49" t="n">
-        <v>6.445139677245978e-07</v>
+        <v>4.033434946491322e-05</v>
       </c>
       <c r="G49" t="n">
         <v>-1.084876209676264</v>
@@ -3367,10 +3367,10 @@
         <v>-0.3563639110360637</v>
       </c>
       <c r="R49" t="n">
-        <v>8.460773354952871e-09</v>
+        <v>1.660214736538174e-05</v>
       </c>
       <c r="S49" t="n">
-        <v>1.870276215305371e-08</v>
+        <v>2.490322104807262e-05</v>
       </c>
       <c r="T49" t="inlineStr">
         <is>
@@ -3396,10 +3396,10 @@
         <v>-0.3257983458008429</v>
       </c>
       <c r="E50" t="n">
-        <v>4.398029969151889e-10</v>
+        <v>9.160237910241471e-10</v>
       </c>
       <c r="F50" t="n">
-        <v>1.531165989260287e-09</v>
+        <v>4.100296969346183e-09</v>
       </c>
       <c r="G50" t="n">
         <v>-1.098108830659307</v>
@@ -3435,10 +3435,10 @@
         <v>-0.4472366428811658</v>
       </c>
       <c r="R50" t="n">
-        <v>1.464077515411452e-13</v>
+        <v>1.369424915744769e-13</v>
       </c>
       <c r="S50" t="n">
-        <v>4.730096588252382e-13</v>
+        <v>4.424295881636946e-13</v>
       </c>
       <c r="T50" t="inlineStr">
         <is>
@@ -3464,10 +3464,10 @@
         <v>-0.2968306861611412</v>
       </c>
       <c r="E51" t="n">
-        <v>0.0165864233862047</v>
+        <v>0.018628508217588</v>
       </c>
       <c r="F51" t="n">
-        <v>0.0187846240759426</v>
+        <v>0.0221655667399148</v>
       </c>
       <c r="G51" t="n">
         <v>-1.194925027264708</v>
@@ -3503,10 +3503,10 @@
         <v>-0.3863390538494</v>
       </c>
       <c r="R51" t="n">
-        <v>0.0089402703325077</v>
+        <v>0.0099951257958896</v>
       </c>
       <c r="S51" t="n">
-        <v>0.0098813514201401</v>
+        <v>0.0107639816263426</v>
       </c>
       <c r="T51" t="inlineStr">
         <is>
@@ -3532,10 +3532,10 @@
         <v>-0.3899630345464017</v>
       </c>
       <c r="E52" t="n">
-        <v>1.214124744033309e-06</v>
+        <v>1.973131190712182e-05</v>
       </c>
       <c r="F52" t="n">
-        <v>2.428249488066618e-06</v>
+        <v>3.785190447488675e-05</v>
       </c>
       <c r="G52" t="n">
         <v>-1.134767216750626</v>
@@ -3584,10 +3584,10 @@
         <v>-0.2057466474024407</v>
       </c>
       <c r="E53" t="n">
-        <v>0.0076473869843637</v>
+        <v>0.0066984208150368</v>
       </c>
       <c r="F53" t="n">
-        <v>0.009335771123768599</v>
+        <v>0.008284888902808599</v>
       </c>
       <c r="G53" t="n">
         <v>-1.108807893958623</v>
@@ -3623,10 +3623,10 @@
         <v>-0.350039338621643</v>
       </c>
       <c r="R53" t="n">
-        <v>9.429593499497854e-05</v>
+        <v>1.887169658373822e-05</v>
       </c>
       <c r="S53" t="n">
-        <v>0.0001237634146809</v>
+        <v>2.733142263851742e-05</v>
       </c>
       <c r="T53" t="inlineStr">
         <is>
@@ -3652,10 +3652,10 @@
         <v>-0.3679674866580253</v>
       </c>
       <c r="E54" t="n">
-        <v>0.0063423310909463</v>
+        <v>0.0004270012418018</v>
       </c>
       <c r="F54" t="n">
-        <v>0.007844462138801999</v>
+        <v>0.0006473889795059</v>
       </c>
       <c r="G54" t="n">
         <v>-1.656290751490781</v>
@@ -3704,10 +3704,10 @@
         <v>-0.3381930384959687</v>
       </c>
       <c r="E55" t="n">
-        <v>0.0014621264034239</v>
+        <v>0.0011745750544174</v>
       </c>
       <c r="F55" t="n">
-        <v>0.0019088872489145</v>
+        <v>0.0016236772811064</v>
       </c>
       <c r="G55" t="n">
         <v>-1.861901919664883</v>
@@ -3743,10 +3743,10 @@
         <v>-0.4441849152303856</v>
       </c>
       <c r="R55" t="n">
-        <v>0.0003230363820293</v>
+        <v>0.0001731019230502</v>
       </c>
       <c r="S55" t="n">
-        <v>0.0003990449425068</v>
+        <v>0.0002203115384275</v>
       </c>
       <c r="T55" t="inlineStr">
         <is>
@@ -3772,10 +3772,10 @@
         <v>-0.2244823712045364</v>
       </c>
       <c r="E56" t="n">
-        <v>0.0058440679493856</v>
+        <v>0.0022288038693353</v>
       </c>
       <c r="F56" t="n">
-        <v>0.0073245651632299</v>
+        <v>0.0029098272738544</v>
       </c>
       <c r="G56" t="n">
         <v>-1.283242500875942</v>
@@ -3811,10 +3811,10 @@
         <v>-0.4088222439671773</v>
       </c>
       <c r="R56" t="n">
-        <v>2.664139000888552e-05</v>
+        <v>1.284999115877519e-05</v>
       </c>
       <c r="S56" t="n">
-        <v>3.858408208183421e-05</v>
+        <v>1.998887513587252e-05</v>
       </c>
       <c r="T56" t="inlineStr">
         <is>
@@ -3840,10 +3840,10 @@
         <v>-0.6858605628042763</v>
       </c>
       <c r="E57" t="n">
-        <v>5.375366681084805e-12</v>
+        <v>1.748971427201253e-17</v>
       </c>
       <c r="F57" t="n">
-        <v>2.105351950091549e-11</v>
+        <v>2.74005523594863e-16</v>
       </c>
       <c r="G57" t="n">
         <v>-1.811098652249668</v>
@@ -3892,10 +3892,10 @@
         <v>-0.3162175777192162</v>
       </c>
       <c r="E58" t="n">
-        <v>1.162462502063463e-06</v>
+        <v>1.356518031392875e-05</v>
       </c>
       <c r="F58" t="n">
-        <v>2.375466852042729e-06</v>
+        <v>2.713036062785749e-05</v>
       </c>
       <c r="G58" t="n">
         <v>-1.219805078787887</v>
@@ -3931,10 +3931,10 @@
         <v>-0.5526040868847748</v>
       </c>
       <c r="R58" t="n">
-        <v>1.374573448524384e-13</v>
+        <v>1.616667441532216e-15</v>
       </c>
       <c r="S58" t="n">
-        <v>4.730096588252382e-13</v>
+        <v>7.544448060483675e-15</v>
       </c>
       <c r="T58" t="inlineStr">
         <is>
@@ -3960,10 +3960,10 @@
         <v>-0.5032675785908065</v>
       </c>
       <c r="E59" t="n">
-        <v>7.080631664356068e-16</v>
+        <v>8.051250769623751e-15</v>
       </c>
       <c r="F59" t="n">
-        <v>4.437195842996469e-15</v>
+        <v>7.568175723446326e-14</v>
       </c>
       <c r="G59" t="n">
         <v>-1.196017737896068</v>
@@ -3999,10 +3999,10 @@
         <v>-0.7478292865875198</v>
       </c>
       <c r="R59" t="n">
-        <v>4.584952706748103e-25</v>
+        <v>3.457049441515893e-28</v>
       </c>
       <c r="S59" t="n">
-        <v>3.209466894723673e-24</v>
+        <v>1.451960765436675e-26</v>
       </c>
       <c r="T59" t="inlineStr">
         <is>
@@ -4028,10 +4028,10 @@
         <v>-0.3612908731320999</v>
       </c>
       <c r="E60" t="n">
-        <v>1.592564136721469e-09</v>
+        <v>6.558509497102431e-09</v>
       </c>
       <c r="F60" t="n">
-        <v>5.162104443166141e-09</v>
+        <v>2.465999570910515e-08</v>
       </c>
       <c r="G60" t="n">
         <v>-1.085801676852166</v>
@@ -4080,10 +4080,10 @@
         <v>-0.2073314783927149</v>
       </c>
       <c r="E61" t="n">
-        <v>0.030420349847232</v>
+        <v>0.0194321514087153</v>
       </c>
       <c r="F61" t="n">
-        <v>0.033250149833021</v>
+        <v>0.0228327779052404</v>
       </c>
       <c r="G61" t="n">
         <v>-1.505100079515383</v>
@@ -4119,10 +4119,10 @@
         <v>-0.4811393899392877</v>
       </c>
       <c r="R61" t="n">
-        <v>3.034127803667951e-05</v>
+        <v>5.307715140098073e-05</v>
       </c>
       <c r="S61" t="n">
-        <v>4.247778925135131e-05</v>
+        <v>7.430801196137302e-05</v>
       </c>
       <c r="T61" t="inlineStr">
         <is>
@@ -4148,10 +4148,10 @@
         <v>-0.3043424817073953</v>
       </c>
       <c r="E62" t="n">
-        <v>0.0015322460691748</v>
+        <v>0.0009960809687460999</v>
       </c>
       <c r="F62" t="n">
-        <v>0.0019730291849648</v>
+        <v>0.0013974867322706</v>
       </c>
       <c r="G62" t="n">
         <v>-1.079861899639728</v>
@@ -4200,10 +4200,10 @@
         <v>-0.0297734376483427</v>
       </c>
       <c r="E63" t="n">
-        <v>0.7773861784358157</v>
+        <v>0.7683365810333102</v>
       </c>
       <c r="F63" t="n">
-        <v>0.7773861784358157</v>
+        <v>0.7683365810333102</v>
       </c>
       <c r="G63" t="n">
         <v>-1.310266817725494</v>
@@ -4239,10 +4239,10 @@
         <v>-0.3093407583952859</v>
       </c>
       <c r="R63" t="n">
-        <v>0.0136879440488612</v>
+        <v>0.0153648291520804</v>
       </c>
       <c r="S63" t="n">
-        <v>0.0147408628218505</v>
+        <v>0.0161330706096844</v>
       </c>
       <c r="T63" t="inlineStr">
         <is>
@@ -4268,10 +4268,10 @@
         <v>-0.3030134467842733</v>
       </c>
       <c r="E64" t="n">
-        <v>0.0125803902232771</v>
+        <v>0.0234844573876647</v>
       </c>
       <c r="F64" t="n">
-        <v>0.0147819585123505</v>
+        <v>0.0262802261242914</v>
       </c>
       <c r="G64" t="n">
         <v>-1.086130185369127</v>
@@ -4320,10 +4320,10 @@
         <v>-0.3397029307464672</v>
       </c>
       <c r="E65" t="n">
-        <v>0.0002463815997421</v>
+        <v>3.446779858617107e-05</v>
       </c>
       <c r="F65" t="n">
-        <v>0.0003456697071008</v>
+        <v>6.11315673037751e-05</v>
       </c>
       <c r="G65" t="n">
         <v>-1.408545036658453</v>
@@ -4372,10 +4372,10 @@
         <v>-0.4099896224645262</v>
       </c>
       <c r="E66" t="n">
-        <v>0.0001249660657188</v>
+        <v>0.0014033399044715</v>
       </c>
       <c r="F66" t="n">
-        <v>0.0001864573044058</v>
+        <v>0.001884485014576</v>
       </c>
       <c r="G66" t="n">
         <v>-1.652638001425365</v>
@@ -4424,10 +4424,10 @@
         <v>-0.3414793540009962</v>
       </c>
       <c r="E67" t="n">
-        <v>9.41170290157365e-07</v>
+        <v>9.941421964319609e-08</v>
       </c>
       <c r="F67" t="n">
-        <v>2.010681983518007e-06</v>
+        <v>2.831798983775888e-07</v>
       </c>
       <c r="G67" t="n">
         <v>-1.129221555732847</v>
@@ -4463,10 +4463,10 @@
         <v>-0.5663813965520188</v>
       </c>
       <c r="R67" t="n">
-        <v>2.408446490320979e-12</v>
+        <v>6.798605460419096e-19</v>
       </c>
       <c r="S67" t="n">
-        <v>6.743650172898739e-12</v>
+        <v>4.759023822293368e-18</v>
       </c>
       <c r="T67" t="inlineStr">
         <is>
@@ -4492,10 +4492,10 @@
         <v>-0.4604913766449164</v>
       </c>
       <c r="E68" t="n">
-        <v>6.257121900727413e-09</v>
+        <v>1.06547172101218e-15</v>
       </c>
       <c r="F68" t="n">
-        <v>1.960564862227923e-08</v>
+        <v>1.251929272189311e-14</v>
       </c>
       <c r="G68" t="n">
         <v>-1.563064365592713</v>
@@ -4544,10 +4544,10 @@
         <v>-0.1141118928139242</v>
       </c>
       <c r="E69" t="n">
-        <v>0.1314110825595688</v>
+        <v>0.0876706225411233</v>
       </c>
       <c r="F69" t="n">
-        <v>0.1372515751177718</v>
+        <v>0.0915670946540621</v>
       </c>
       <c r="G69" t="n">
         <v>-1.009147192525029</v>
@@ -4583,10 +4583,10 @@
         <v>-0.4331177593834895</v>
       </c>
       <c r="R69" t="n">
-        <v>8.677271797084175e-07</v>
+        <v>3.918095767028573e-08</v>
       </c>
       <c r="S69" t="n">
-        <v>1.614892606349051e-06</v>
+        <v>8.228001110760003e-08</v>
       </c>
       <c r="T69" t="inlineStr">
         <is>
@@ -4612,10 +4612,10 @@
         <v>-0.3740772267246099</v>
       </c>
       <c r="E70" t="n">
-        <v>7.295166160730784e-07</v>
+        <v>3.909173724075955e-05</v>
       </c>
       <c r="F70" t="n">
-        <v>1.632727664544509e-06</v>
+        <v>6.804857964132216e-05</v>
       </c>
       <c r="G70" t="n">
         <v>-1.359704319580233</v>
@@ -4651,10 +4651,10 @@
         <v>-0.6019968834116127</v>
       </c>
       <c r="R70" t="n">
-        <v>1.141964057282769e-11</v>
+        <v>6.541128137227055e-09</v>
       </c>
       <c r="S70" t="n">
-        <v>2.997655650367268e-11</v>
+        <v>1.616043422138449e-08</v>
       </c>
       <c r="T70" t="inlineStr">
         <is>
@@ -4680,10 +4680,10 @@
         <v>-0.4646554691796039</v>
       </c>
       <c r="E71" t="n">
-        <v>5.981291938388129e-05</v>
+        <v>9.381843885760794e-08</v>
       </c>
       <c r="F71" t="n">
-        <v>9.370690703474736e-05</v>
+        <v>2.755916641442234e-07</v>
       </c>
       <c r="G71" t="n">
         <v>-1.564790426979868</v>
@@ -4732,10 +4732,10 @@
         <v>-0.5151457640163549</v>
       </c>
       <c r="E72" t="n">
-        <v>1.320554696871435e-07</v>
+        <v>2.142159027025679e-11</v>
       </c>
       <c r="F72" t="n">
-        <v>3.354922743403105e-07</v>
+        <v>1.18448793259067e-10</v>
       </c>
       <c r="G72" t="n">
         <v>-1.763019369775018</v>
@@ -4784,10 +4784,10 @@
         <v>-0.3190578285775493</v>
       </c>
       <c r="E73" t="n">
-        <v>0.0122832924611463</v>
+        <v>0.0032311745148042</v>
       </c>
       <c r="F73" t="n">
-        <v>0.0146155631816171</v>
+        <v>0.0041044649242107</v>
       </c>
       <c r="G73" t="n">
         <v>-1.630902550954251</v>
@@ -4836,10 +4836,10 @@
         <v>-0.2128638797981655</v>
       </c>
       <c r="E74" t="n">
-        <v>0.008052595716382401</v>
+        <v>0.01656540670027</v>
       </c>
       <c r="F74" t="n">
-        <v>0.0097044102223069</v>
+        <v>0.0199634388439151</v>
       </c>
       <c r="G74" t="n">
         <v>-1.180753668104172</v>
@@ -4875,10 +4875,10 @@
         <v>-0.5418172229337404</v>
       </c>
       <c r="R74" t="n">
-        <v>5.261576504866698e-09</v>
+        <v>3.073991959829152e-08</v>
       </c>
       <c r="S74" t="n">
-        <v>1.227701184468896e-08</v>
+        <v>6.7951401217276e-08</v>
       </c>
       <c r="T74" t="inlineStr">
         <is>
@@ -4904,10 +4904,10 @@
         <v>-0.4734237073794558</v>
       </c>
       <c r="E75" t="n">
-        <v>8.66467112002183e-09</v>
+        <v>1.980925935396086e-06</v>
       </c>
       <c r="F75" t="n">
-        <v>2.545247141506413e-08</v>
+        <v>4.541635071395904e-06</v>
       </c>
       <c r="G75" t="n">
         <v>-1.307557453374142</v>
@@ -4956,10 +4956,10 @@
         <v>-0.0906861366649319</v>
       </c>
       <c r="E76" t="n">
-        <v>0.389179032142069</v>
+        <v>0.4074733176059139</v>
       </c>
       <c r="F76" t="n">
-        <v>0.3976394458842879</v>
+        <v>0.4163314332060424</v>
       </c>
       <c r="G76" t="n">
         <v>-1.529616875876403</v>
@@ -4995,10 +4995,10 @@
         <v>-0.2707626825603527</v>
       </c>
       <c r="R76" t="n">
-        <v>0.0322417922244778</v>
+        <v>0.0298991351432502</v>
       </c>
       <c r="S76" t="n">
-        <v>0.0322417922244778</v>
+        <v>0.0306283823418661</v>
       </c>
       <c r="T76" t="inlineStr">
         <is>
@@ -5024,10 +5024,10 @@
         <v>-0.1240508910173154</v>
       </c>
       <c r="E77" t="n">
-        <v>0.1918507930290651</v>
+        <v>0.1880901252314683</v>
       </c>
       <c r="F77" t="n">
-        <v>0.1981755444476057</v>
+        <v>0.1942908985907475</v>
       </c>
       <c r="G77" t="n">
         <v>-1.040453467812631</v>
@@ -5063,10 +5063,10 @@
         <v>-0.3282586976917905</v>
       </c>
       <c r="R77" t="n">
-        <v>0.0033890974353183</v>
+        <v>0.0024871075692936</v>
       </c>
       <c r="S77" t="n">
-        <v>0.0039539470078713</v>
+        <v>0.0027489083660614</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
@@ -5092,10 +5092,10 @@
         <v>-0.3834885473728106</v>
       </c>
       <c r="E78" t="n">
-        <v>2.142856641492325e-05</v>
+        <v>5.80430072579744e-08</v>
       </c>
       <c r="F78" t="n">
-        <v>3.66233680545961e-05</v>
+        <v>1.818680894083198e-07</v>
       </c>
       <c r="G78" t="n">
         <v>-1.244820848235848</v>
@@ -5131,10 +5131,10 @@
         <v>-0.5289056492437357</v>
       </c>
       <c r="R78" t="n">
-        <v>8.843459510959089e-07</v>
+        <v>7.696236371668819e-11</v>
       </c>
       <c r="S78" t="n">
-        <v>1.614892606349051e-06</v>
+        <v>2.154946184067269e-10</v>
       </c>
       <c r="T78" t="inlineStr">
         <is>
@@ -5160,10 +5160,10 @@
         <v>-0.2709097624984234</v>
       </c>
       <c r="E79" t="n">
-        <v>5.380048833393938e-05</v>
+        <v>0.0001037631276661</v>
       </c>
       <c r="F79" t="n">
-        <v>8.571603226085258e-05</v>
+        <v>0.0001681678275967</v>
       </c>
       <c r="G79" t="n">
         <v>-1.280779954131551</v>
@@ -5199,10 +5199,10 @@
         <v>-0.3492822908622425</v>
       </c>
       <c r="R79" t="n">
-        <v>8.945287336425944e-06</v>
+        <v>0.0001224784620978</v>
       </c>
       <c r="S79" t="n">
-        <v>1.391489141221813e-05</v>
+        <v>0.0001659385615518</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
@@ -5228,10 +5228,10 @@
         <v>-0.6092265479979961</v>
       </c>
       <c r="E80" t="n">
-        <v>3.314403007253767e-15</v>
+        <v>6.361732945199844e-07</v>
       </c>
       <c r="F80" t="n">
-        <v>1.639757277272916e-14</v>
+        <v>1.616224045537257e-06</v>
       </c>
       <c r="G80" t="n">
         <v>-1.252704173171887</v>
@@ -5280,10 +5280,10 @@
         <v>-0.0332848358903953</v>
       </c>
       <c r="E81" t="n">
-        <v>0.6074587448528381</v>
+        <v>0.6245519301711997</v>
       </c>
       <c r="F81" t="n">
-        <v>0.6139905593136213</v>
+        <v>0.6312675423235782</v>
       </c>
       <c r="G81" t="n">
         <v>-1.012028474786338</v>
@@ -5319,10 +5319,10 @@
         <v>-0.298367592746348</v>
       </c>
       <c r="R81" t="n">
-        <v>7.988464419551615e-05</v>
+        <v>0.0001922792376518</v>
       </c>
       <c r="S81" t="n">
-        <v>0.0001082308082648</v>
+        <v>0.000237521411217</v>
       </c>
       <c r="T81" t="inlineStr">
         <is>
@@ -5348,10 +5348,10 @@
         <v>-0.4700288525771587</v>
       </c>
       <c r="E82" t="n">
-        <v>3.619375649710779e-05</v>
+        <v>5.314734465338386e-06</v>
       </c>
       <c r="F82" t="n">
-        <v>6.075380554871665e-05</v>
+        <v>1.110188977204018e-05</v>
       </c>
       <c r="G82" t="n">
         <v>-2.004145108267159</v>
@@ -5400,10 +5400,10 @@
         <v>-0.2687038524514541</v>
       </c>
       <c r="E83" t="n">
-        <v>0.0002699866717892</v>
+        <v>0.0007186710692564</v>
       </c>
       <c r="F83" t="n">
-        <v>0.0003732168698262</v>
+        <v>0.0010235618259106</v>
       </c>
       <c r="G83" t="n">
         <v>-1.022686670993109</v>
@@ -5452,10 +5452,10 @@
         <v>-0.4298802981883268</v>
       </c>
       <c r="E84" t="n">
-        <v>0.0001733636815278</v>
+        <v>0.000603900605509</v>
       </c>
       <c r="F84" t="n">
-        <v>0.0002469119100547</v>
+        <v>0.0008733331833514</v>
       </c>
       <c r="G84" t="n">
         <v>-1.509491831303903</v>
@@ -5504,10 +5504,10 @@
         <v>-0.4081568690676349</v>
       </c>
       <c r="E85" t="n">
-        <v>7.29595575325603e-06</v>
+        <v>2.468061709110689e-06</v>
       </c>
       <c r="F85" t="n">
-        <v>1.399632328175646e-05</v>
+        <v>5.395297689683833e-06</v>
       </c>
       <c r="G85" t="n">
         <v>-1.7196491711041</v>
@@ -5543,10 +5543,10 @@
         <v>-0.8422389450349099</v>
       </c>
       <c r="R85" t="n">
-        <v>3.647563243378535e-15</v>
+        <v>4.159058187575141e-12</v>
       </c>
       <c r="S85" t="n">
-        <v>1.531976562218985e-14</v>
+        <v>1.247717456272542e-11</v>
       </c>
       <c r="T85" t="inlineStr">
         <is>
@@ -5572,10 +5572,10 @@
         <v>-0.319483951446612</v>
       </c>
       <c r="E86" t="n">
-        <v>7.281066572836062e-05</v>
+        <v>0.0013919691910065</v>
       </c>
       <c r="F86" t="n">
-        <v>0.0001122000422699</v>
+        <v>0.001884485014576</v>
       </c>
       <c r="G86" t="n">
         <v>-1.054139446371316</v>
@@ -5624,10 +5624,10 @@
         <v>-0.4215633484812767</v>
       </c>
       <c r="E87" t="n">
-        <v>8.942619651372594e-06</v>
+        <v>3.021844750617789e-06</v>
       </c>
       <c r="F87" t="n">
-        <v>1.648247543586321e-05</v>
+        <v>6.455759239956186e-06</v>
       </c>
       <c r="G87" t="n">
         <v>-1.078034845268306</v>
@@ -5676,10 +5676,10 @@
         <v>-0.3485900680439985</v>
       </c>
       <c r="E88" t="n">
-        <v>1.335944354365068e-05</v>
+        <v>0.0005873125437006</v>
       </c>
       <c r="F88" t="n">
-        <v>2.4149763328907e-05</v>
+        <v>0.0008626152985602</v>
       </c>
       <c r="G88" t="n">
         <v>-1.131728656938623</v>
@@ -5728,10 +5728,10 @@
         <v>-0.3296539752833525</v>
       </c>
       <c r="E89" t="n">
-        <v>1.855517055171026e-05</v>
+        <v>0.0025825601054011</v>
       </c>
       <c r="F89" t="n">
-        <v>3.290917041246727e-05</v>
+        <v>0.0033254883549</v>
       </c>
       <c r="G89" t="n">
         <v>-1.019572670762451</v>
@@ -5767,10 +5767,10 @@
         <v>-0.6448054359569048</v>
       </c>
       <c r="R89" t="n">
-        <v>8.596751161173015e-14</v>
+        <v>1.241833679628212e-08</v>
       </c>
       <c r="S89" t="n">
-        <v>3.282395897902423e-13</v>
+        <v>2.897611919132496e-08</v>
       </c>
       <c r="T89" t="inlineStr">
         <is>
@@ -5796,10 +5796,10 @@
         <v>-0.4030554970745703</v>
       </c>
       <c r="E90" t="n">
-        <v>4.705664043335697e-08</v>
+        <v>8.682988446007943e-07</v>
       </c>
       <c r="F90" t="n">
-        <v>1.228701166870987e-07</v>
+        <v>2.147897141907228e-06</v>
       </c>
       <c r="G90" t="n">
         <v>-1.6822690149032</v>
@@ -5835,10 +5835,10 @@
         <v>-0.763783179065633</v>
       </c>
       <c r="R90" t="n">
-        <v>1.691064228158077e-19</v>
+        <v>2.214758723924796e-17</v>
       </c>
       <c r="S90" t="n">
-        <v>8.878087197829902e-19</v>
+        <v>1.328855234354878e-16</v>
       </c>
       <c r="T90" t="inlineStr">
         <is>
@@ -5864,10 +5864,10 @@
         <v>-0.1724510025955488</v>
       </c>
       <c r="E91" t="n">
-        <v>0.0451193928128345</v>
+        <v>0.0245213356369539</v>
       </c>
       <c r="F91" t="n">
-        <v>0.0481957150500732</v>
+        <v>0.0271177123514549</v>
       </c>
       <c r="G91" t="n">
         <v>-1.088930411191174</v>
@@ -5903,10 +5903,10 @@
         <v>-0.4852044571786227</v>
       </c>
       <c r="R91" t="n">
-        <v>1.888785179370901e-06</v>
+        <v>1.455699063525099e-07</v>
       </c>
       <c r="S91" t="n">
-        <v>3.173159101343113e-06</v>
+        <v>2.833791847279979e-07</v>
       </c>
       <c r="T91" t="inlineStr">
         <is>
@@ -5932,10 +5932,10 @@
         <v>-0.4964450259015118</v>
       </c>
       <c r="E92" t="n">
-        <v>3.164132424307008e-14</v>
+        <v>1.935094414929326e-08</v>
       </c>
       <c r="F92" t="n">
-        <v>1.416325942308852e-13</v>
+        <v>6.736995370494689e-08</v>
       </c>
       <c r="G92" t="n">
         <v>-1.163983595429531</v>
@@ -5984,10 +5984,10 @@
         <v>-0.5335887791486136</v>
       </c>
       <c r="E93" t="n">
-        <v>9.852205662885487e-07</v>
+        <v>1.003714827195982e-11</v>
       </c>
       <c r="F93" t="n">
-        <v>2.058016294024968e-06</v>
+        <v>6.289946250428156e-11</v>
       </c>
       <c r="G93" t="n">
         <v>-2.569111507472138</v>
@@ -6036,10 +6036,10 @@
         <v>-0.5048474904163017</v>
       </c>
       <c r="E94" t="n">
-        <v>0.0007320770079146</v>
+        <v>3.139695156275106e-07</v>
       </c>
       <c r="F94" t="n">
-        <v>0.0009830748391996</v>
+        <v>8.198092908051665e-07</v>
       </c>
       <c r="G94" t="n">
         <v>-1.459898022277849</v>
@@ -6088,10 +6088,10 @@
         <v>-0.3934983649132454</v>
       </c>
       <c r="E95" t="n">
-        <v>3.541373412708916e-06</v>
+        <v>1.761869364729693e-06</v>
       </c>
       <c r="F95" t="n">
-        <v>6.935189599888294e-06</v>
+        <v>4.140393007114778e-06</v>
       </c>
       <c r="G95" t="n">
         <v>-1.488230514489267</v>

</xml_diff>